<commit_message>
Hapus teks spesifik perusahaan pada template Excel
</commit_message>
<xml_diff>
--- a/Template_Dashboard.xlsx
+++ b/Template_Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pkt841-my.sharepoint.com/personal/deptkpmrpkt_pkt841_onmicrosoft_com/Documents/Manajemen Risiko Korporasi/PROJECT/Proyek/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365mic-my.sharepoint.com/personal/ipanjez_365mic_onmicrosoft_com/Documents/Learn/Coding/Dashboard Proyek Soda Ash/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38E74821-C745-4135-9F3A-19FA6098A12F}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{901E0FE3-4737-4F4F-849C-FBD9465FF939}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -516,9 +516,6 @@
     <t>EXECUTIVE ACTION TRACKER — DIREKSI / PROJECT STEERING COMMITTEE (PSC)</t>
   </si>
   <si>
-    <t>Soda Ash Project PT Pupuk Kalimantan Timur — diperbarui setiap periode pelaporan bulanan. Kategori Level mengikuti klasifikasi 5-tingkat Pedoman Manajemen Risiko PKT.</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -552,9 +549,6 @@
     <t>Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A.</t>
   </si>
   <si>
-    <t>VP Proyek Soda Ash &amp; SVP Pengembangan Portofolio</t>
-  </si>
-  <si>
     <t>Mencegah kegagalan penyelesaian proyek bersamaan, mengamankan target COD Maret 2028, melindungi NPV sebesar USD 77,60 Juta.</t>
   </si>
   <si>
@@ -567,12 +561,6 @@
     <t>Finansial — Moderate to High</t>
   </si>
   <si>
-    <t>Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Pupuk Indonesia (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</t>
-  </si>
-  <si>
-    <t>Direktur Utama PKT &amp; SVP Keuangan</t>
-  </si>
-  <si>
     <t>Melindungi penyelesaian gardu kelistrikan dan fasilitas tie-in, menghindari denda klaim tambahan dari EPC-A.</t>
   </si>
   <si>
@@ -588,9 +576,6 @@
     <t>Lobi aktif dan koordinasi dengan Kementerian Perindustrian serta Kementerian Kelautan dan Perikanan guna mengamankan alokasi kuota impor tahunan setahun sebelum operasional dimulai, merujuk Perpres No.17/2025.</t>
   </si>
   <si>
-    <t>Direktur Utama PKT &amp; SVP Pengembangan Portofolio</t>
-  </si>
-  <si>
     <t>Menghindari penghentian operasional akibat kekosongan bahan baku; menghemat potensi kerugian EBITDA Rp 137 Miliar/kuartal.</t>
   </si>
   <si>
@@ -606,9 +591,6 @@
     <t>Menginstruksikan Kompartemen Keuangan mengimplementasikan strategi hedging valas (forward/opsi) bekerja sama dengan bank BUMN nasional untuk mengunci porsi sisa pembayaran dalam USD.</t>
   </si>
   <si>
-    <t>Direktur Keuangan PKT</t>
-  </si>
-  <si>
     <t>Mengeliminasi risiko pembengkakan biaya investasi riil akibat depresiasi rupiah; mengamankan ambang batas investasi USD 297,67 Juta.</t>
   </si>
   <si>
@@ -621,18 +603,9 @@
     <t>Regulasi — Moderate</t>
   </si>
   <si>
-    <t>Membentuk tim percepatan perizinan internal untuk koordinasi harian dengan DLH Kota Bontang dan Dinas PUPR Provinsi Kaltim guna mempercepat adendum dokumen lingkungan di lahan sengketa.</t>
-  </si>
-  <si>
-    <t>VP Hukum &amp; Humas PKT</t>
-  </si>
-  <si>
     <t>Mencegah keterlambatan masa efektif konstruksi fisik; menghemat opportunity cost of capital senilai Rp 500 Juta/bulan.</t>
   </si>
   <si>
-    <t>Sumber tata kelola: Risk Register Soda Ash 2025; kerangka Gate Review &amp; FID PT Pertamina (Persero); Weighted Project Top Risk (Financial Materiality 40%, Strategic Impact 30%, Life Cycle Phase 15%, Financial Health Impact 10%, Baseline Risk Complexity 5%). Level risiko mengikuti klasifikasi 5-tingkat Pedoman Manajemen Risiko PKT: Low / Low to Moderate / Moderate / Moderate to High / High.</t>
-  </si>
-  <si>
     <t>DINAMIKA PERGERAKAN RISIKO (BULAN BERJALAN)</t>
   </si>
   <si>
@@ -681,9 +654,6 @@
     <t>Score / Level</t>
   </si>
   <si>
-    <t>PROJECT RISK &amp; HEALTH DASHBOARD  -  SODA ASH PROJECT  PT PUPUK KALIMANTAN TIMUR (PKT)</t>
-  </si>
-  <si>
     <t>PANEL A - PROJECT HEALTH OVERVIEW (Retrospective Performance)</t>
   </si>
   <si>
@@ -886,9 +856,6 @@
   </si>
   <si>
     <t>REFERENSI FORMULA &amp; AMBANG BATAS (THRESHOLD) — PROJECT RISK &amp; HEALTH DASHBOARD</t>
-  </si>
-  <si>
-    <t>Soda Ash Project PT Pupuk Kalimantan Timur | Sumber: Standarisasi Eksekutif Project Risk &amp; Health Dashboard (Studi Kelayakan Deloitte; Risk Register Soda Ash 2025) &amp; Benchmark PT Pertamina (Persero) - Direktorat Manajemen Risiko / Permen BUMN No.02/2023</t>
   </si>
   <si>
     <t>1. LIMA PILAR KESEHATAN PROYEK (PROJECT HEALTH) &amp; FORMULA</t>
@@ -946,27 +913,18 @@
     <t>SRI = S (Wi x Si)</t>
   </si>
   <si>
-    <t>Risk Register Soda Ash - Pengelompokan Tahapan Pekerjaan Proyek (2025)</t>
-  </si>
-  <si>
     <t>4 parameter tertimbang pelaksanaan EPC</t>
   </si>
   <si>
     <t>PEI = S (Pj x Wj)</t>
   </si>
   <si>
-    <t>Risk Register Soda Ash 2025; praktik EPC Progress-S-Curve industri</t>
-  </si>
-  <si>
     <t>5 parameter tertimbang kesiapan komersial</t>
   </si>
   <si>
     <t>CRI = S (Wk x Sk)</t>
   </si>
   <si>
-    <t>Risk Register Soda Ash 2025</t>
-  </si>
-  <si>
     <t>PHS = (FinancialScore x 0,20) + (ScheduleScore x 0,20) + (SRI x 0,20) + (PEI x 0,20) + (CRI x 0,20)</t>
   </si>
   <si>
@@ -1186,9 +1144,6 @@
     <t>6. KRITERIA LIKELIHOOD (PROBABILITAS) - MATRIKS RISIKO 5x5</t>
   </si>
   <si>
-    <t>Catatan: kriteria berikut merupakan kriteria standar manajemen risiko (ISO 31000 &amp; benchmark Pertamina RCSA/KRI). Sesuaikan dengan Pedoman Manajemen Risiko PKT resmi apabila tersedia angka baku internal.</t>
-  </si>
-  <si>
     <t>Level (L)</t>
   </si>
   <si>
@@ -1264,9 +1219,6 @@
     <t>Dampak biaya &gt; USD 30 Juta; keterlambatan &gt; 6 bulan atau mengancam kegagalan COD; berdampak pada kelayakan NPV proyek &amp; reputasi korporat.</t>
   </si>
   <si>
-    <t>8. KLASIFIKASI LEVEL RISIKO - 5 TINGKAT (Pedoman Manajemen Risiko PKT)</t>
-  </si>
-  <si>
     <t>Skor Matriks L x C TIDAK lagi dihitung dari perkalian langsung L x C dengan pembagian rentang rata, melainkan menggunakan Tabel Skala Risiko Non-Linear (Skala 1-25) pada bagian 10 di bawah, yang memprioritaskan bobot Consequence (Dampak) dibanding Likelihood (Probabilitas) untuk kombinasi bernilai sama — konsisten dengan pendekatan penentuan level risiko non-linear yang lazim digunakan pada matriks 5x5 ISO 31000:2018 / AS-NZS ISO 31000 dan praktik matriks risiko K3/SMKP BUMN sektor energi-tambang (rujukan pola: Kepdirjen Minerba No.1827.K/30/MEM/2018). Overall Risk Index (skala 0-100, benchmark Pertamina) tetap memakai rentang rata seperti semula.</t>
   </si>
   <si>
@@ -1327,21 +1279,12 @@
     <t>Commercial Risk Index</t>
   </si>
   <si>
-    <t>Pengikatan kontrak offtake, fluktuasi harga soda ash global, tekanan produk impor, kesiapan logistik distribusi hilir, sertifikasi kualitas produk.</t>
-  </si>
-  <si>
     <t>Overall Risk Index = (Supply Risk Index x 0,40) + (Execution Risk Index x 0,40) + (Commercial Risk Index x 0,20)</t>
   </si>
   <si>
-    <t>Sumber benchmark tata kelola risiko: PT Pertamina (Persero) - Direktorat Manajemen Risiko (2nd Line of Defense, Permen BUMN No.02/2023), Komite Tata Kelola Terintegrasi (KTKT), Gate Review/FID, RCSA, KRI, ICT, C-RBDD; PT Biro Klasifikasi Indonesia (Persero) - SK-6/2023 (Risk Appetite berbasis Net Working Capital); klasifikasi 5-tingkat Low/Low to Moderate/Moderate/Moderate to High/High mengikuti nomenklatur Pedoman Manajemen Risiko PKT.</t>
-  </si>
-  <si>
     <t>10. TABEL SKALA RISIKO (RISK RANKING) 5x5 NON-LINEAR &amp; WARNA HEAT MAP</t>
   </si>
   <si>
-    <t>Tabel skala risiko berikut menetapkan urutan (rank) 1-25 untuk setiap 25 kombinasi Likelihood (L) x Consequence (C) sesuai spesifikasi metodologi risiko internal yang ditetapkan Project Control Soda Ash PKT. Berbeda dari perkalian L x C sederhana, urutan ini memberi bobot lebih besar pada Consequence saat terjadi nilai sama, mengikuti kaidah umum non-linear risk ranking pada standar ISO 31000:2018 dan praktik matriks risiko korporasi BUMN. Skala menentukan posisi &amp; warna sel pada Risk Profile Heat Map di sheet Dashboard.</t>
-  </si>
-  <si>
     <t>Key (L x10 + C)</t>
   </si>
   <si>
@@ -1372,9 +1315,6 @@
     <t>#E06666</t>
   </si>
   <si>
-    <t>Sumber/Referensi Tabel Skala: metodologi non-linear risk ranking ISO 31000:2018 (klausul 5.4.3 - penentuan level risiko); praktik matriks 5x5 K3/SMKP BUMN sektor energi &amp; tambang; disesuaikan dengan nomenklatur 5-tingkat Pedoman Manajemen Risiko PKT (Low / Low to Moderate / Moderate / Moderate to High / High).</t>
-  </si>
-  <si>
     <t>11. METODOLOGI EARLY WARNING SYSTEM (EWS) — 3 STATUS (AMAN / WASPADA / BAHAYA)</t>
   </si>
   <si>
@@ -1450,9 +1390,6 @@
     <t>Risiko sangat tinggi (proyek terhenti)</t>
   </si>
   <si>
-    <t>Mengukur tingkat risiko komersial &amp; pemasaran produk soda ash</t>
-  </si>
-  <si>
     <t>Offtake agreement, strategi pemasaran, kesiapan distribusi, kualifikasi produk, persaingan impor</t>
   </si>
   <si>
@@ -1465,12 +1402,6 @@
     <t>Formula Overall Risk Index = (Supply Risk Index × 0,4) + (Execution Risk Index × 0,4) + (Commercial Risk Index × 0,2)</t>
   </si>
   <si>
-    <t>13. KLASIFIKASI JUMLAH REGISTER RISIKO AKTIF (5 TINGKAT PKT)</t>
-  </si>
-  <si>
-    <t>Setiap risiko dalam register diklasifikasi berdasarkan Skala Risiko Non-Linear 5x5 (bagian 10) ke dalam 5 tingkat risiko PKT:</t>
-  </si>
-  <si>
     <t>Rentang Skala (1-25)</t>
   </si>
   <si>
@@ -1630,9 +1561,6 @@
     <t>Overall Risk Level (5 Tingkat, formula)</t>
   </si>
   <si>
-    <t>6. REGISTER RISIKO AKTIF — Jumlah Risiko per 5 Tingkat PKT</t>
-  </si>
-  <si>
     <t>7. STATUS MITIGASI &amp; DINAMIKA PERGERAKAN RISIKO (BULAN BERJALAN)</t>
   </si>
   <si>
@@ -1739,6 +1667,78 @@
   </si>
   <si>
     <t>Regulatory Readiness</t>
+  </si>
+  <si>
+    <t>PROJECT RISK &amp; HEALTH DASHBOARD  -  Proyek X PROJECT  Perusahaan X (Perusahaan X)</t>
+  </si>
+  <si>
+    <t>Risk Register Proyek X - Pengelompokan Tahapan Pekerjaan Proyek (2025)</t>
+  </si>
+  <si>
+    <t>Risk Register Proyek X 2025; praktik EPC Progress-S-Curve industri</t>
+  </si>
+  <si>
+    <t>Risk Register Proyek X 2025</t>
+  </si>
+  <si>
+    <t>Pengikatan kontrak offtake, fluktuasi harga Proyek X global, tekanan produk impor, kesiapan logistik distribusi hilir, sertifikasi kualitas produk.</t>
+  </si>
+  <si>
+    <t>Mengukur tingkat risiko komersial &amp; pemasaran produk Proyek X</t>
+  </si>
+  <si>
+    <t>Proyek X Project Perusahaan X | Sumber: Standarisasi Eksekutif Project Risk &amp; Health Dashboard (Studi Kelayakan Deloitte; Risk Register Proyek X 2025) &amp; Benchmark PT Pertamina (Persero) - Direktorat Manajemen Risiko / Permen BUMN No.02/2023</t>
+  </si>
+  <si>
+    <t>Catatan: kriteria berikut merupakan kriteria standar manajemen risiko (ISO 31000 &amp; benchmark Pertamina RCSA/KRI). Sesuaikan dengan Pedoman Manajemen Risiko Perusahaan X resmi apabila tersedia angka baku internal.</t>
+  </si>
+  <si>
+    <t>8. KLASIFIKASI LEVEL RISIKO - 5 TINGKAT (Pedoman Manajemen Risiko Perusahaan X)</t>
+  </si>
+  <si>
+    <t>Sumber benchmark tata kelola risiko: PT Pertamina (Persero) - Direktorat Manajemen Risiko (2nd Line of Defense, Permen BUMN No.02/2023), Komite Tata Kelola Terintegrasi (KTKT), Gate Review/FID, RCSA, KRI, ICT, C-RBDD; PT Biro Klasifikasi Indonesia (Persero) - SK-6/2023 (Risk Appetite berbasis Net Working Capital); klasifikasi 5-tingkat Low/Low to Moderate/Moderate/Moderate to High/High mengikuti nomenklatur Pedoman Manajemen Risiko Perusahaan X.</t>
+  </si>
+  <si>
+    <t>Tabel skala risiko berikut menetapkan urutan (rank) 1-25 untuk setiap 25 kombinasi Likelihood (L) x Consequence (C) sesuai spesifikasi metodologi risiko internal yang ditetapkan Project Control Proyek X Perusahaan X. Berbeda dari perkalian L x C sederhana, urutan ini memberi bobot lebih besar pada Consequence saat terjadi nilai sama, mengikuti kaidah umum non-linear risk ranking pada standar ISO 31000:2018 dan praktik matriks risiko korporasi BUMN. Skala menentukan posisi &amp; warna sel pada Risk Profile Heat Map di sheet Dashboard.</t>
+  </si>
+  <si>
+    <t>Sumber/Referensi Tabel Skala: metodologi non-linear risk ranking ISO 31000:2018 (klausul 5.4.3 - penentuan level risiko); praktik matriks 5x5 K3/SMKP BUMN sektor energi &amp; tambang; disesuaikan dengan nomenklatur 5-tingkat Pedoman Manajemen Risiko Perusahaan X (Low / Low to Moderate / Moderate / Moderate to High / High).</t>
+  </si>
+  <si>
+    <t>13. KLASIFIKASI JUMLAH REGISTER RISIKO AKTIF (5 TINGKAT Perusahaan X)</t>
+  </si>
+  <si>
+    <t>Setiap risiko dalam register diklasifikasi berdasarkan Skala Risiko Non-Linear 5x5 (bagian 10) ke dalam 5 tingkat risiko Perusahaan X:</t>
+  </si>
+  <si>
+    <t>6. REGISTER RISIKO AKTIF — Jumlah Risiko per 5 Tingkat Perusahaan X</t>
+  </si>
+  <si>
+    <t>VP Proyek Proyek X &amp; SVP Pengembangan Portofolio</t>
+  </si>
+  <si>
+    <t>Proyek X Project Perusahaan X — diperbarui setiap periode pelaporan bulanan. Kategori Level mengikuti klasifikasi 5-tingkat Pedoman Manajemen Risiko Perusahaan X.</t>
+  </si>
+  <si>
+    <t>Direktur Utama Perusahaan X &amp; SVP Keuangan</t>
+  </si>
+  <si>
+    <t>Direktur Utama Perusahaan X &amp; SVP Pengembangan Portofolio</t>
+  </si>
+  <si>
+    <t>Direktur Keuangan Perusahaan X</t>
+  </si>
+  <si>
+    <t>VP Hukum &amp; Humas Perusahaan X</t>
+  </si>
+  <si>
+    <t>Sumber tata kelola: Risk Register Proyek X 2025; kerangka Gate Review &amp; FID PT Pertamina (Persero); Weighted Project Top Risk (Financial Materiality 40%, Strategic Impact 30%, Life Cycle Phase 15%, Financial Health Impact 10%, Baseline Risk Complexity 5%). Level risiko mengikuti klasifikasi 5-tingkat Pedoman Manajemen Risiko Perusahaan X: Low / Low to Moderate / Moderate / Moderate to High / High.</t>
+  </si>
+  <si>
+    <t>Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Perusahaan Induk X (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</t>
+  </si>
+  <si>
+    <t>Membentuk tim percepatan perizinan internal untuk koordinasi harian dengan DLH Kota X dan Dinas PUPR Provinsi Provinsi X guna mempercepat adendum dokumen lingkungan di lahan sengketa.</t>
   </si>
 </sst>
 </file>
@@ -2763,207 +2763,207 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3382,8 +3382,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="167" t="s">
-        <v>56</v>
+      <c r="B1" s="182" t="s">
+        <v>384</v>
       </c>
       <c r="C1" s="116"/>
       <c r="D1" s="116"/>
@@ -3408,9 +3408,9 @@
       <c r="W1" s="118"/>
     </row>
     <row r="2" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="186" t="str">
+      <c r="B2" s="152" t="str">
         <f ca="1">"Reporting Period: "&amp;Input_Bulanan!D5&amp;"   |   Status: "&amp;Input_Bulanan!F5&amp;"   |   Dicetak: "&amp;TEXT(TODAY(),"DD-MM-YYYY")</f>
-        <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 17-07-2026</v>
+        <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 18-07-2026</v>
       </c>
       <c r="C2" s="114"/>
       <c r="D2" s="114"/>
@@ -3436,8 +3436,8 @@
     </row>
     <row r="3" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="138" t="s">
-        <v>57</v>
+      <c r="B4" s="153" t="s">
+        <v>47</v>
       </c>
       <c r="C4" s="116"/>
       <c r="D4" s="116"/>
@@ -3449,8 +3449,8 @@
       <c r="J4" s="116"/>
       <c r="K4" s="116"/>
       <c r="L4" s="118"/>
-      <c r="M4" s="138" t="s">
-        <v>58</v>
+      <c r="M4" s="153" t="s">
+        <v>48</v>
       </c>
       <c r="N4" s="116"/>
       <c r="O4" s="116"/>
@@ -3464,30 +3464,30 @@
       <c r="W4" s="118"/>
     </row>
     <row r="5" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="152" t="s">
-        <v>59</v>
+      <c r="B5" s="162" t="s">
+        <v>49</v>
       </c>
       <c r="C5" s="116"/>
       <c r="D5" s="116"/>
       <c r="E5" s="116"/>
       <c r="F5" s="118"/>
-      <c r="G5" s="152" t="s">
-        <v>60</v>
+      <c r="G5" s="162" t="s">
+        <v>50</v>
       </c>
       <c r="H5" s="116"/>
       <c r="I5" s="116"/>
       <c r="J5" s="116"/>
       <c r="K5" s="116"/>
       <c r="L5" s="118"/>
-      <c r="M5" s="152" t="s">
-        <v>61</v>
+      <c r="M5" s="162" t="s">
+        <v>51</v>
       </c>
       <c r="N5" s="116"/>
       <c r="O5" s="116"/>
       <c r="P5" s="116"/>
       <c r="Q5" s="118"/>
-      <c r="R5" s="188" t="s">
-        <v>62</v>
+      <c r="R5" s="147" t="s">
+        <v>52</v>
       </c>
       <c r="S5" s="116"/>
       <c r="T5" s="116"/>
@@ -3496,35 +3496,35 @@
       <c r="W5" s="118"/>
     </row>
     <row r="6" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="154">
+      <c r="B6" s="192">
         <f>((IF(Input_Bulanan!D11&gt;=1,100,Input_Bulanan!D11*100)*0.2)+(IF(Input_Bulanan!D13&gt;=1,100,Input_Bulanan!D13*100)*0.2)+(Input_Bulanan!D22*100*0.2)+(Input_Bulanan!D29*100*0.2)+(Input_Bulanan!D38*100*0.2))/100</f>
         <v>0.69100000000000006</v>
       </c>
-      <c r="C6" s="142"/>
-      <c r="D6" s="142"/>
-      <c r="E6" s="142"/>
-      <c r="F6" s="143"/>
-      <c r="G6" s="173" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="142"/>
-      <c r="I6" s="142"/>
-      <c r="J6" s="142"/>
-      <c r="K6" s="148">
+      <c r="C6" s="156"/>
+      <c r="D6" s="156"/>
+      <c r="E6" s="156"/>
+      <c r="F6" s="142"/>
+      <c r="G6" s="160" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="156"/>
+      <c r="I6" s="156"/>
+      <c r="J6" s="156"/>
+      <c r="K6" s="141">
         <f>Input_Bulanan!D22</f>
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="L6" s="143"/>
-      <c r="M6" s="187" t="str">
+      <c r="L6" s="142"/>
+      <c r="M6" s="155" t="str">
         <f>Input_Bulanan!D45</f>
         <v>Moderate</v>
       </c>
-      <c r="N6" s="142"/>
-      <c r="O6" s="142"/>
-      <c r="P6" s="142"/>
-      <c r="Q6" s="143"/>
+      <c r="N6" s="156"/>
+      <c r="O6" s="156"/>
+      <c r="P6" s="156"/>
+      <c r="Q6" s="142"/>
       <c r="R6" s="1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="S6" s="2" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
@@ -3548,24 +3548,24 @@
       </c>
     </row>
     <row r="7" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="155"/>
+      <c r="B7" s="157"/>
       <c r="C7" s="114"/>
       <c r="D7" s="114"/>
       <c r="E7" s="114"/>
-      <c r="F7" s="156"/>
-      <c r="G7" s="144"/>
-      <c r="H7" s="145"/>
-      <c r="I7" s="145"/>
-      <c r="J7" s="145"/>
-      <c r="K7" s="145"/>
-      <c r="L7" s="146"/>
-      <c r="M7" s="155"/>
+      <c r="F7" s="158"/>
+      <c r="G7" s="159"/>
+      <c r="H7" s="143"/>
+      <c r="I7" s="143"/>
+      <c r="J7" s="143"/>
+      <c r="K7" s="143"/>
+      <c r="L7" s="144"/>
+      <c r="M7" s="157"/>
       <c r="N7" s="114"/>
       <c r="O7" s="114"/>
       <c r="P7" s="114"/>
-      <c r="Q7" s="156"/>
+      <c r="Q7" s="158"/>
       <c r="R7" s="1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="S7" s="3" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
@@ -3589,29 +3589,29 @@
       </c>
     </row>
     <row r="8" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="155"/>
+      <c r="B8" s="157"/>
       <c r="C8" s="114"/>
       <c r="D8" s="114"/>
       <c r="E8" s="114"/>
-      <c r="F8" s="156"/>
-      <c r="G8" s="173" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="142"/>
-      <c r="I8" s="142"/>
-      <c r="J8" s="142"/>
-      <c r="K8" s="148">
+      <c r="F8" s="158"/>
+      <c r="G8" s="160" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="156"/>
+      <c r="I8" s="156"/>
+      <c r="J8" s="156"/>
+      <c r="K8" s="141">
         <f>Input_Bulanan!D29</f>
         <v>0.76800000000000002</v>
       </c>
-      <c r="L8" s="143"/>
-      <c r="M8" s="155"/>
+      <c r="L8" s="142"/>
+      <c r="M8" s="157"/>
       <c r="N8" s="114"/>
       <c r="O8" s="114"/>
       <c r="P8" s="114"/>
-      <c r="Q8" s="156"/>
+      <c r="Q8" s="158"/>
       <c r="R8" s="1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="S8" s="5" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
@@ -3635,24 +3635,24 @@
       </c>
     </row>
     <row r="9" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="144"/>
-      <c r="C9" s="145"/>
-      <c r="D9" s="145"/>
-      <c r="E9" s="145"/>
-      <c r="F9" s="146"/>
-      <c r="G9" s="144"/>
-      <c r="H9" s="145"/>
-      <c r="I9" s="145"/>
-      <c r="J9" s="145"/>
-      <c r="K9" s="145"/>
-      <c r="L9" s="146"/>
-      <c r="M9" s="144"/>
-      <c r="N9" s="145"/>
-      <c r="O9" s="145"/>
-      <c r="P9" s="145"/>
-      <c r="Q9" s="146"/>
+      <c r="B9" s="159"/>
+      <c r="C9" s="143"/>
+      <c r="D9" s="143"/>
+      <c r="E9" s="143"/>
+      <c r="F9" s="144"/>
+      <c r="G9" s="159"/>
+      <c r="H9" s="143"/>
+      <c r="I9" s="143"/>
+      <c r="J9" s="143"/>
+      <c r="K9" s="143"/>
+      <c r="L9" s="144"/>
+      <c r="M9" s="159"/>
+      <c r="N9" s="143"/>
+      <c r="O9" s="143"/>
+      <c r="P9" s="143"/>
+      <c r="Q9" s="144"/>
       <c r="R9" s="1" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="S9" s="6" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
@@ -3676,35 +3676,35 @@
       </c>
     </row>
     <row r="10" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="141" t="str">
+      <c r="B10" s="191" t="str">
         <f>IF(B6&gt;=0.9,"HIJAU - SEHAT",IF(B6&gt;=0.75,"KUNING - PANTAU",IF(B6&gt;=0.6,"ORANYE - WASPADA","MERAH - KRITIS")))</f>
         <v>ORANYE - WASPADA</v>
       </c>
-      <c r="C10" s="142"/>
-      <c r="D10" s="142"/>
-      <c r="E10" s="142"/>
-      <c r="F10" s="143"/>
-      <c r="G10" s="173" t="s">
-        <v>69</v>
-      </c>
-      <c r="H10" s="142"/>
-      <c r="I10" s="142"/>
-      <c r="J10" s="142"/>
-      <c r="K10" s="148">
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="142"/>
+      <c r="G10" s="160" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="156"/>
+      <c r="I10" s="156"/>
+      <c r="J10" s="156"/>
+      <c r="K10" s="141">
         <f>Input_Bulanan!D38</f>
         <v>0.62</v>
       </c>
-      <c r="L10" s="143"/>
-      <c r="M10" s="175" t="str">
+      <c r="L10" s="142"/>
+      <c r="M10" s="168" t="str">
         <f>"Skor Komposit: "&amp;TEXT(Input_Bulanan!D44,"0,00")&amp;" / 100"</f>
         <v>Skor Komposit: 45,80 / 100</v>
       </c>
-      <c r="N10" s="142"/>
-      <c r="O10" s="142"/>
-      <c r="P10" s="142"/>
-      <c r="Q10" s="143"/>
+      <c r="N10" s="156"/>
+      <c r="O10" s="156"/>
+      <c r="P10" s="156"/>
+      <c r="Q10" s="142"/>
       <c r="R10" s="1" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="S10" s="6" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
@@ -3728,24 +3728,24 @@
       </c>
     </row>
     <row r="11" spans="2:23" ht="12" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="144"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="146"/>
-      <c r="G11" s="144"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="145"/>
-      <c r="L11" s="146"/>
-      <c r="M11" s="144"/>
-      <c r="N11" s="145"/>
-      <c r="O11" s="145"/>
-      <c r="P11" s="145"/>
-      <c r="Q11" s="146"/>
+      <c r="B11" s="159"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="144"/>
+      <c r="G11" s="159"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="143"/>
+      <c r="L11" s="144"/>
+      <c r="M11" s="159"/>
+      <c r="N11" s="143"/>
+      <c r="O11" s="143"/>
+      <c r="P11" s="143"/>
+      <c r="Q11" s="144"/>
       <c r="R11" s="7" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="S11" s="8">
         <v>1</v>
@@ -3764,30 +3764,30 @@
       </c>
     </row>
     <row r="12" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="152" t="s">
-        <v>72</v>
+      <c r="B12" s="162" t="s">
+        <v>62</v>
       </c>
       <c r="C12" s="116"/>
       <c r="D12" s="116"/>
       <c r="E12" s="116"/>
       <c r="F12" s="118"/>
-      <c r="G12" s="152" t="s">
-        <v>73</v>
+      <c r="G12" s="162" t="s">
+        <v>63</v>
       </c>
       <c r="H12" s="116"/>
       <c r="I12" s="116"/>
       <c r="J12" s="116"/>
       <c r="K12" s="116"/>
       <c r="L12" s="118"/>
-      <c r="M12" s="152" t="s">
-        <v>74</v>
+      <c r="M12" s="162" t="s">
+        <v>64</v>
       </c>
       <c r="N12" s="116"/>
       <c r="O12" s="116"/>
       <c r="P12" s="116"/>
       <c r="Q12" s="118"/>
-      <c r="R12" s="152" t="s">
-        <v>75</v>
+      <c r="R12" s="162" t="s">
+        <v>65</v>
       </c>
       <c r="S12" s="116"/>
       <c r="T12" s="116"/>
@@ -3796,33 +3796,33 @@
       <c r="W12" s="118"/>
     </row>
     <row r="13" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="151" t="s">
-        <v>76</v>
+      <c r="B13" s="148" t="s">
+        <v>66</v>
       </c>
       <c r="C13" s="116"/>
       <c r="D13" s="118"/>
-      <c r="E13" s="171">
+      <c r="E13" s="165">
         <f>Input_Bulanan!D11</f>
         <v>1</v>
       </c>
       <c r="F13" s="118"/>
-      <c r="G13" s="139" t="s">
-        <v>77</v>
+      <c r="G13" s="187" t="s">
+        <v>67</v>
       </c>
       <c r="H13" s="116"/>
       <c r="I13" s="118"/>
-      <c r="J13" s="162">
+      <c r="J13" s="167">
         <f>Input_Bulanan!D8</f>
         <v>100</v>
       </c>
       <c r="K13" s="116"/>
       <c r="L13" s="118"/>
-      <c r="M13" s="157" t="s">
-        <v>78</v>
+      <c r="M13" s="161" t="s">
+        <v>68</v>
       </c>
       <c r="N13" s="116"/>
       <c r="O13" s="118"/>
-      <c r="P13" s="161">
+      <c r="P13" s="188">
         <f>Input_Bulanan!D48</f>
         <v>5</v>
       </c>
@@ -3831,7 +3831,7 @@
         <f>Input_Bulanan!C74</f>
         <v>C1</v>
       </c>
-      <c r="S13" s="160" t="str">
+      <c r="S13" s="172" t="str">
         <f>Input_Bulanan!D74&amp;"  |  L="&amp;Input_Bulanan!F74&amp;", C="&amp;Input_Bulanan!G74&amp;", Skala="&amp;Input_Bulanan!H74&amp;" -&gt; "&amp;Input_Bulanan!I74</f>
         <v>Salt Supply Disruption (gangguan pasokan garam industri)  |  L=4, C=5, Skala=24 -&gt; High</v>
       </c>
@@ -3841,33 +3841,33 @@
       <c r="W13" s="116"/>
     </row>
     <row r="14" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="151" t="s">
-        <v>79</v>
+      <c r="B14" s="148" t="s">
+        <v>69</v>
       </c>
       <c r="C14" s="116"/>
       <c r="D14" s="118"/>
-      <c r="E14" s="171">
+      <c r="E14" s="165">
         <f>Input_Bulanan!D13</f>
         <v>1</v>
       </c>
       <c r="F14" s="118"/>
-      <c r="G14" s="139" t="s">
-        <v>80</v>
+      <c r="G14" s="187" t="s">
+        <v>70</v>
       </c>
       <c r="H14" s="116"/>
       <c r="I14" s="118"/>
-      <c r="J14" s="162">
+      <c r="J14" s="167">
         <f>Input_Bulanan!D9</f>
         <v>100</v>
       </c>
       <c r="K14" s="116"/>
       <c r="L14" s="118"/>
-      <c r="M14" s="157" t="s">
-        <v>81</v>
+      <c r="M14" s="161" t="s">
+        <v>71</v>
       </c>
       <c r="N14" s="116"/>
       <c r="O14" s="118"/>
-      <c r="P14" s="176">
+      <c r="P14" s="170">
         <f>Input_Bulanan!D49</f>
         <v>11</v>
       </c>
@@ -3876,7 +3876,7 @@
         <f>Input_Bulanan!C75</f>
         <v>C2</v>
       </c>
-      <c r="S14" s="160" t="str">
+      <c r="S14" s="172" t="str">
         <f>Input_Bulanan!D75&amp;"  |  L="&amp;Input_Bulanan!F75&amp;", C="&amp;Input_Bulanan!G75&amp;", Skala="&amp;Input_Bulanan!H75&amp;" -&gt; "&amp;Input_Bulanan!I75</f>
         <v>Commissioning Delay (keterlambatan commissioning)  |  L=5, C=5, Skala=25 -&gt; High</v>
       </c>
@@ -3886,33 +3886,33 @@
       <c r="W14" s="116"/>
     </row>
     <row r="15" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="151" t="s">
-        <v>82</v>
+      <c r="B15" s="148" t="s">
+        <v>72</v>
       </c>
       <c r="C15" s="116"/>
       <c r="D15" s="118"/>
-      <c r="E15" s="174">
+      <c r="E15" s="150">
         <f>Input_Bulanan!D12</f>
         <v>0</v>
       </c>
       <c r="F15" s="118"/>
-      <c r="G15" s="139" t="s">
-        <v>83</v>
+      <c r="G15" s="187" t="s">
+        <v>73</v>
       </c>
       <c r="H15" s="116"/>
       <c r="I15" s="118"/>
-      <c r="J15" s="162">
+      <c r="J15" s="167">
         <f>Input_Bulanan!D10</f>
         <v>100</v>
       </c>
       <c r="K15" s="116"/>
       <c r="L15" s="118"/>
-      <c r="M15" s="157" t="s">
-        <v>84</v>
+      <c r="M15" s="161" t="s">
+        <v>74</v>
       </c>
       <c r="N15" s="116"/>
       <c r="O15" s="118"/>
-      <c r="P15" s="163">
+      <c r="P15" s="189">
         <f>Input_Bulanan!D50</f>
         <v>18</v>
       </c>
@@ -3921,7 +3921,7 @@
         <f>Input_Bulanan!C76</f>
         <v>C3</v>
       </c>
-      <c r="S15" s="160" t="str">
+      <c r="S15" s="172" t="str">
         <f>Input_Bulanan!D76&amp;"  |  L="&amp;Input_Bulanan!F76&amp;", C="&amp;Input_Bulanan!G76&amp;", Skala="&amp;Input_Bulanan!H76&amp;" -&gt; "&amp;Input_Bulanan!I76</f>
         <v>EPC Interface Issue (isu EPC interface lintas kontraktor)  |  L=4, C=4, Skala=19 -&gt; Moderate to High</v>
       </c>
@@ -3931,30 +3931,30 @@
       <c r="W15" s="116"/>
     </row>
     <row r="16" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="151" t="s">
-        <v>85</v>
+      <c r="B16" s="148" t="s">
+        <v>75</v>
       </c>
       <c r="C16" s="116"/>
       <c r="D16" s="118"/>
-      <c r="E16" s="174">
+      <c r="E16" s="150">
         <f>Input_Bulanan!D14</f>
         <v>0</v>
       </c>
       <c r="F16" s="118"/>
-      <c r="G16" s="192" t="s">
-        <v>86</v>
+      <c r="G16" s="151" t="s">
+        <v>76</v>
       </c>
       <c r="H16" s="116"/>
       <c r="I16" s="116"/>
       <c r="J16" s="116"/>
       <c r="K16" s="116"/>
       <c r="L16" s="118"/>
-      <c r="M16" s="157" t="s">
-        <v>87</v>
+      <c r="M16" s="161" t="s">
+        <v>77</v>
       </c>
       <c r="N16" s="116"/>
       <c r="O16" s="118"/>
-      <c r="P16" s="191">
+      <c r="P16" s="145">
         <f>Input_Bulanan!D51</f>
         <v>4</v>
       </c>
@@ -3963,7 +3963,7 @@
         <f>Input_Bulanan!C77</f>
         <v>C4</v>
       </c>
-      <c r="S16" s="160" t="str">
+      <c r="S16" s="172" t="str">
         <f>Input_Bulanan!D77&amp;"  |  L="&amp;Input_Bulanan!F77&amp;", C="&amp;Input_Bulanan!G77&amp;", Skala="&amp;Input_Bulanan!H77&amp;" -&gt; "&amp;Input_Bulanan!I77</f>
         <v>Long Lead Equipment (keterlambatan peralatan utama)  |  L=3, C=3, Skala=13 -&gt; Moderate</v>
       </c>
@@ -3974,12 +3974,12 @@
     </row>
     <row r="17" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="L17" s="106"/>
-      <c r="M17" s="157" t="s">
-        <v>88</v>
+      <c r="M17" s="161" t="s">
+        <v>78</v>
       </c>
       <c r="N17" s="116"/>
       <c r="O17" s="118"/>
-      <c r="P17" s="191">
+      <c r="P17" s="145">
         <f>Input_Bulanan!D52</f>
         <v>3</v>
       </c>
@@ -3987,11 +3987,11 @@
     </row>
     <row r="18" spans="2:23" x14ac:dyDescent="0.45">
       <c r="M18" s="105" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="N18" s="103"/>
       <c r="O18" s="104"/>
-      <c r="P18" s="190">
+      <c r="P18" s="149">
         <f>Input_Bulanan!D53</f>
         <v>41</v>
       </c>
@@ -4016,21 +4016,21 @@
       <c r="Q19" s="114"/>
     </row>
     <row r="20" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="177" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="178"/>
-      <c r="D20" s="178"/>
-      <c r="E20" s="178"/>
-      <c r="F20" s="178"/>
-      <c r="G20" s="178"/>
-      <c r="H20" s="178"/>
-      <c r="I20" s="178"/>
-      <c r="J20" s="178"/>
-      <c r="K20" s="178"/>
-      <c r="L20" s="179"/>
-      <c r="M20" s="172" t="s">
-        <v>91</v>
+      <c r="B20" s="173" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="174"/>
+      <c r="D20" s="174"/>
+      <c r="E20" s="174"/>
+      <c r="F20" s="174"/>
+      <c r="G20" s="174"/>
+      <c r="H20" s="174"/>
+      <c r="I20" s="174"/>
+      <c r="J20" s="174"/>
+      <c r="K20" s="174"/>
+      <c r="L20" s="175"/>
+      <c r="M20" s="186" t="s">
+        <v>81</v>
       </c>
       <c r="N20" s="116"/>
       <c r="O20" s="116"/>
@@ -4038,92 +4038,92 @@
       <c r="Q20" s="118"/>
     </row>
     <row r="21" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="180"/>
-      <c r="C21" s="181"/>
-      <c r="D21" s="181"/>
-      <c r="E21" s="181"/>
-      <c r="F21" s="181"/>
-      <c r="G21" s="181"/>
-      <c r="H21" s="181"/>
-      <c r="I21" s="181"/>
-      <c r="J21" s="181"/>
-      <c r="K21" s="181"/>
-      <c r="L21" s="182"/>
-      <c r="M21" s="151" t="s">
-        <v>92</v>
+      <c r="B21" s="176"/>
+      <c r="C21" s="177"/>
+      <c r="D21" s="177"/>
+      <c r="E21" s="177"/>
+      <c r="F21" s="177"/>
+      <c r="G21" s="177"/>
+      <c r="H21" s="177"/>
+      <c r="I21" s="177"/>
+      <c r="J21" s="177"/>
+      <c r="K21" s="177"/>
+      <c r="L21" s="178"/>
+      <c r="M21" s="148" t="s">
+        <v>82</v>
       </c>
       <c r="N21" s="116"/>
       <c r="O21" s="118"/>
-      <c r="P21" s="149">
+      <c r="P21" s="163">
         <f>Input_Bulanan!D56</f>
         <v>0.82</v>
       </c>
       <c r="Q21" s="118"/>
     </row>
     <row r="22" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="180"/>
-      <c r="C22" s="181"/>
-      <c r="D22" s="181"/>
-      <c r="E22" s="181"/>
-      <c r="F22" s="181"/>
-      <c r="G22" s="181"/>
-      <c r="H22" s="181"/>
-      <c r="I22" s="181"/>
-      <c r="J22" s="181"/>
-      <c r="K22" s="181"/>
-      <c r="L22" s="182"/>
-      <c r="M22" s="151" t="s">
-        <v>93</v>
+      <c r="B22" s="176"/>
+      <c r="C22" s="177"/>
+      <c r="D22" s="177"/>
+      <c r="E22" s="177"/>
+      <c r="F22" s="177"/>
+      <c r="G22" s="177"/>
+      <c r="H22" s="177"/>
+      <c r="I22" s="177"/>
+      <c r="J22" s="177"/>
+      <c r="K22" s="177"/>
+      <c r="L22" s="178"/>
+      <c r="M22" s="148" t="s">
+        <v>83</v>
       </c>
       <c r="N22" s="116"/>
       <c r="O22" s="118"/>
-      <c r="P22" s="149">
+      <c r="P22" s="163">
         <f>Input_Bulanan!D57</f>
         <v>0.18</v>
       </c>
       <c r="Q22" s="118"/>
     </row>
     <row r="23" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="180"/>
-      <c r="C23" s="181"/>
-      <c r="D23" s="181"/>
-      <c r="E23" s="181"/>
-      <c r="F23" s="181"/>
-      <c r="G23" s="181"/>
-      <c r="H23" s="181"/>
-      <c r="I23" s="181"/>
-      <c r="J23" s="181"/>
-      <c r="K23" s="181"/>
-      <c r="L23" s="182"/>
-      <c r="M23" s="151" t="s">
-        <v>94</v>
+      <c r="B23" s="176"/>
+      <c r="C23" s="177"/>
+      <c r="D23" s="177"/>
+      <c r="E23" s="177"/>
+      <c r="F23" s="177"/>
+      <c r="G23" s="177"/>
+      <c r="H23" s="177"/>
+      <c r="I23" s="177"/>
+      <c r="J23" s="177"/>
+      <c r="K23" s="177"/>
+      <c r="L23" s="178"/>
+      <c r="M23" s="148" t="s">
+        <v>84</v>
       </c>
       <c r="N23" s="116"/>
       <c r="O23" s="118"/>
-      <c r="P23" s="149">
+      <c r="P23" s="163">
         <f>Input_Bulanan!D58</f>
         <v>0.76</v>
       </c>
       <c r="Q23" s="118"/>
     </row>
     <row r="24" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="183"/>
-      <c r="C24" s="184"/>
-      <c r="D24" s="184"/>
-      <c r="E24" s="184"/>
-      <c r="F24" s="184"/>
-      <c r="G24" s="184"/>
-      <c r="H24" s="184"/>
-      <c r="I24" s="184"/>
-      <c r="J24" s="184"/>
-      <c r="K24" s="184"/>
-      <c r="L24" s="185"/>
-      <c r="M24" s="151" t="s">
-        <v>95</v>
+      <c r="B24" s="179"/>
+      <c r="C24" s="180"/>
+      <c r="D24" s="180"/>
+      <c r="E24" s="180"/>
+      <c r="F24" s="180"/>
+      <c r="G24" s="180"/>
+      <c r="H24" s="180"/>
+      <c r="I24" s="180"/>
+      <c r="J24" s="180"/>
+      <c r="K24" s="180"/>
+      <c r="L24" s="181"/>
+      <c r="M24" s="148" t="s">
+        <v>85</v>
       </c>
       <c r="N24" s="116"/>
       <c r="O24" s="118"/>
-      <c r="P24" s="168">
+      <c r="P24" s="183">
         <f>Input_Bulanan!D59</f>
         <v>5</v>
       </c>
@@ -4154,8 +4154,8 @@
       <c r="W25" s="114"/>
     </row>
     <row r="26" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="158" t="s">
-        <v>96</v>
+      <c r="B26" s="166" t="s">
+        <v>86</v>
       </c>
       <c r="C26" s="116"/>
       <c r="D26" s="116"/>
@@ -4180,34 +4180,34 @@
       <c r="W26" s="118"/>
     </row>
     <row r="27" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="147" t="s">
-        <v>97</v>
+      <c r="B27" s="164" t="s">
+        <v>87</v>
       </c>
       <c r="C27" s="116"/>
       <c r="D27" s="116"/>
       <c r="E27" s="116"/>
       <c r="F27" s="118"/>
-      <c r="G27" s="147" t="s">
-        <v>98</v>
+      <c r="G27" s="164" t="s">
+        <v>88</v>
       </c>
       <c r="H27" s="116"/>
       <c r="I27" s="116"/>
       <c r="J27" s="118"/>
-      <c r="K27" s="147" t="s">
-        <v>99</v>
+      <c r="K27" s="164" t="s">
+        <v>89</v>
       </c>
       <c r="L27" s="118"/>
       <c r="M27" s="12" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="O27" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="P27" s="147" t="s">
-        <v>103</v>
+        <v>92</v>
+      </c>
+      <c r="P27" s="164" t="s">
+        <v>93</v>
       </c>
       <c r="Q27" s="116"/>
       <c r="R27" s="116"/>
@@ -4218,20 +4218,20 @@
       <c r="W27" s="118"/>
     </row>
     <row r="28" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="139" t="s">
-        <v>104</v>
+      <c r="B28" s="187" t="s">
+        <v>94</v>
       </c>
       <c r="C28" s="116"/>
       <c r="D28" s="116"/>
       <c r="E28" s="116"/>
       <c r="F28" s="118"/>
-      <c r="G28" s="150" t="s">
-        <v>105</v>
+      <c r="G28" s="140" t="s">
+        <v>95</v>
       </c>
       <c r="H28" s="116"/>
       <c r="I28" s="116"/>
       <c r="J28" s="118"/>
-      <c r="K28" s="169">
+      <c r="K28" s="184">
         <f>Input_Bulanan!E63</f>
         <v>24</v>
       </c>
@@ -4248,8 +4248,8 @@
         <f>IF(Input_Bulanan!H63="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P28" s="189" t="s">
-        <v>106</v>
+      <c r="P28" s="139" t="s">
+        <v>96</v>
       </c>
       <c r="Q28" s="116"/>
       <c r="R28" s="116"/>
@@ -4260,20 +4260,20 @@
       <c r="W28" s="118"/>
     </row>
     <row r="29" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="153" t="s">
-        <v>107</v>
+      <c r="B29" s="138" t="s">
+        <v>97</v>
       </c>
       <c r="C29" s="116"/>
       <c r="D29" s="116"/>
       <c r="E29" s="116"/>
       <c r="F29" s="118"/>
-      <c r="G29" s="165" t="s">
-        <v>108</v>
+      <c r="G29" s="171" t="s">
+        <v>98</v>
       </c>
       <c r="H29" s="116"/>
       <c r="I29" s="116"/>
       <c r="J29" s="118"/>
-      <c r="K29" s="140">
+      <c r="K29" s="146">
         <f>Input_Bulanan!E64</f>
         <v>0.73</v>
       </c>
@@ -4290,8 +4290,8 @@
         <f>IF(Input_Bulanan!H64="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P29" s="164" t="s">
-        <v>109</v>
+      <c r="P29" s="169" t="s">
+        <v>99</v>
       </c>
       <c r="Q29" s="116"/>
       <c r="R29" s="116"/>
@@ -4302,20 +4302,20 @@
       <c r="W29" s="118"/>
     </row>
     <row r="30" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="139" t="s">
-        <v>110</v>
+      <c r="B30" s="187" t="s">
+        <v>100</v>
       </c>
       <c r="C30" s="116"/>
       <c r="D30" s="116"/>
       <c r="E30" s="116"/>
       <c r="F30" s="118"/>
-      <c r="G30" s="150" t="s">
-        <v>111</v>
+      <c r="G30" s="140" t="s">
+        <v>101</v>
       </c>
       <c r="H30" s="116"/>
       <c r="I30" s="116"/>
       <c r="J30" s="118"/>
-      <c r="K30" s="170">
+      <c r="K30" s="185">
         <f>Input_Bulanan!E65</f>
         <v>0.94</v>
       </c>
@@ -4332,8 +4332,8 @@
         <f>IF(Input_Bulanan!H65="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P30" s="189" t="s">
-        <v>112</v>
+      <c r="P30" s="139" t="s">
+        <v>102</v>
       </c>
       <c r="Q30" s="116"/>
       <c r="R30" s="116"/>
@@ -4344,20 +4344,20 @@
       <c r="W30" s="118"/>
     </row>
     <row r="31" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="153" t="s">
-        <v>113</v>
+      <c r="B31" s="138" t="s">
+        <v>103</v>
       </c>
       <c r="C31" s="116"/>
       <c r="D31" s="116"/>
       <c r="E31" s="116"/>
       <c r="F31" s="118"/>
-      <c r="G31" s="165" t="s">
-        <v>114</v>
+      <c r="G31" s="171" t="s">
+        <v>104</v>
       </c>
       <c r="H31" s="116"/>
       <c r="I31" s="116"/>
       <c r="J31" s="118"/>
-      <c r="K31" s="140">
+      <c r="K31" s="146">
         <f>Input_Bulanan!E66</f>
         <v>0.75</v>
       </c>
@@ -4374,8 +4374,8 @@
         <f>IF(Input_Bulanan!H66="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P31" s="164" t="s">
-        <v>115</v>
+      <c r="P31" s="169" t="s">
+        <v>105</v>
       </c>
       <c r="Q31" s="116"/>
       <c r="R31" s="116"/>
@@ -4386,20 +4386,20 @@
       <c r="W31" s="118"/>
     </row>
     <row r="32" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="139" t="s">
-        <v>116</v>
+      <c r="B32" s="187" t="s">
+        <v>106</v>
       </c>
       <c r="C32" s="116"/>
       <c r="D32" s="116"/>
       <c r="E32" s="116"/>
       <c r="F32" s="118"/>
-      <c r="G32" s="150" t="s">
-        <v>117</v>
+      <c r="G32" s="140" t="s">
+        <v>107</v>
       </c>
       <c r="H32" s="116"/>
       <c r="I32" s="116"/>
       <c r="J32" s="118"/>
-      <c r="K32" s="166">
+      <c r="K32" s="190">
         <f>Input_Bulanan!E67</f>
         <v>0.42</v>
       </c>
@@ -4416,8 +4416,8 @@
         <f>IF(Input_Bulanan!H67="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P32" s="189" t="s">
-        <v>118</v>
+      <c r="P32" s="139" t="s">
+        <v>108</v>
       </c>
       <c r="Q32" s="116"/>
       <c r="R32" s="116"/>
@@ -4428,20 +4428,20 @@
       <c r="W32" s="118"/>
     </row>
     <row r="33" spans="2:23" x14ac:dyDescent="0.45">
-      <c r="B33" s="153" t="s">
-        <v>119</v>
+      <c r="B33" s="138" t="s">
+        <v>109</v>
       </c>
       <c r="C33" s="116"/>
       <c r="D33" s="116"/>
       <c r="E33" s="116"/>
       <c r="F33" s="118"/>
-      <c r="G33" s="165" t="s">
-        <v>120</v>
+      <c r="G33" s="171" t="s">
+        <v>110</v>
       </c>
       <c r="H33" s="116"/>
       <c r="I33" s="116"/>
       <c r="J33" s="118"/>
-      <c r="K33" s="140">
+      <c r="K33" s="146">
         <f>Input_Bulanan!E68</f>
         <v>0.4</v>
       </c>
@@ -4458,8 +4458,8 @@
         <f>IF(Input_Bulanan!H68="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P33" s="164" t="s">
-        <v>121</v>
+      <c r="P33" s="169" t="s">
+        <v>111</v>
       </c>
       <c r="Q33" s="116"/>
       <c r="R33" s="116"/>
@@ -4494,8 +4494,8 @@
       <c r="W34" s="114"/>
     </row>
     <row r="35" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="158" t="s">
-        <v>122</v>
+      <c r="B35" s="166" t="s">
+        <v>112</v>
       </c>
       <c r="C35" s="116"/>
       <c r="D35" s="116"/>
@@ -4520,9 +4520,9 @@
       <c r="W35" s="118"/>
     </row>
     <row r="36" spans="2:23" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="159" t="str">
+      <c r="B36" s="154" t="str">
         <f>"Prioritas 1—2: [1] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 1), Risk_Action_Tracker!Z$6:Z$15, 0)) &amp; " · [2] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 2), Risk_Action_Tracker!Z$6:Z$15, 0))</f>
-        <v>Prioritas 1—2: [1] Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A. · [2] Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Pupuk Indonesia (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</v>
+        <v>Prioritas 1—2: [1] Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A. · [2] Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Perusahaan Induk X (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</v>
       </c>
       <c r="C36" s="116"/>
       <c r="D36" s="116"/>
@@ -4547,8 +4547,8 @@
       <c r="W36" s="118"/>
     </row>
     <row r="37" spans="2:23" ht="42.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="159" t="s">
-        <v>123</v>
+      <c r="B37" s="154" t="s">
+        <v>113</v>
       </c>
       <c r="C37" s="116"/>
       <c r="D37" s="116"/>
@@ -4574,24 +4574,70 @@
     </row>
   </sheetData>
   <mergeCells count="98">
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="P30:W30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="K6:L7"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P32:W32"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="P28:W28"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B19:L19"/>
-    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="M4:W4"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="B10:F11"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="G5:L5"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="B6:F9"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="B36:W36"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="K10:L11"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="S15:W15"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P31:W31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="P29:W29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B35:W35"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="B25:W25"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="M10:Q11"/>
+    <mergeCell ref="P33:W33"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="S16:W16"/>
+    <mergeCell ref="B20:L24"/>
     <mergeCell ref="B2:W2"/>
     <mergeCell ref="B34:W34"/>
     <mergeCell ref="B4:L4"/>
@@ -4608,70 +4654,24 @@
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="P23:Q23"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B35:W35"/>
-    <mergeCell ref="G6:J7"/>
-    <mergeCell ref="B25:W25"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="M10:Q11"/>
-    <mergeCell ref="P33:W33"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="S16:W16"/>
-    <mergeCell ref="B20:L24"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="P29:W29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="R12:W12"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B36:W36"/>
-    <mergeCell ref="S14:W14"/>
-    <mergeCell ref="K10:L11"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="S15:W15"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="P31:W31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M4:W4"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="B10:F11"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="G5:L5"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="B6:F9"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="P28:W28"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="P30:W30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="K6:L7"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P32:W32"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:F11">
     <cfRule type="expression" dxfId="11" priority="2">
@@ -4742,7 +4742,7 @@
   <sheetData>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="13" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -4750,8 +4750,8 @@
       <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="133" t="s">
-        <v>125</v>
+      <c r="A3" s="125" t="s">
+        <v>390</v>
       </c>
       <c r="B3" s="114"/>
       <c r="C3" s="114"/>
@@ -4759,8 +4759,8 @@
       <c r="E3" s="114"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="117" t="s">
-        <v>126</v>
+      <c r="A5" s="120" t="s">
+        <v>115</v>
       </c>
       <c r="B5" s="116"/>
       <c r="C5" s="116"/>
@@ -4769,104 +4769,104 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="14" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="15" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="19" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D8" s="110">
         <v>0.2</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="15" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="D9" s="110">
         <v>0.2</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>143</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="19" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="D10" s="110">
         <v>0.2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>146</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="15" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D11" s="110">
         <v>0.2</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>149</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4874,12 +4874,12 @@
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="22" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="137" t="s">
-        <v>150</v>
+      <c r="A14" s="113" t="s">
+        <v>136</v>
       </c>
       <c r="B14" s="114"/>
       <c r="C14" s="114"/>
@@ -4887,8 +4887,8 @@
       <c r="E14" s="114"/>
     </row>
     <row r="15" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="113" t="s">
-        <v>151</v>
+      <c r="A15" s="134" t="s">
+        <v>137</v>
       </c>
       <c r="B15" s="114"/>
       <c r="C15" s="114"/>
@@ -4896,8 +4896,8 @@
       <c r="E15" s="114"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="117" t="s">
-        <v>152</v>
+      <c r="A17" s="120" t="s">
+        <v>138</v>
       </c>
       <c r="B17" s="116"/>
       <c r="C17" s="116"/>
@@ -4906,85 +4906,85 @@
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="14" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="C18" s="135" t="s">
-        <v>154</v>
+        <v>139</v>
+      </c>
+      <c r="C18" s="122" t="s">
+        <v>140</v>
       </c>
       <c r="D18" s="116"/>
       <c r="E18" s="118"/>
     </row>
     <row r="19" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="15" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="B19" s="110">
         <v>0.25</v>
       </c>
-      <c r="C19" s="122" t="s">
-        <v>156</v>
+      <c r="C19" s="123" t="s">
+        <v>142</v>
       </c>
       <c r="D19" s="116"/>
       <c r="E19" s="116"/>
     </row>
     <row r="20" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="19" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="B20" s="111">
         <v>0.2</v>
       </c>
       <c r="C20" s="115" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="D20" s="116"/>
       <c r="E20" s="116"/>
     </row>
     <row r="21" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="15" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="B21" s="110">
         <v>0.2</v>
       </c>
-      <c r="C21" s="122" t="s">
-        <v>160</v>
+      <c r="C21" s="123" t="s">
+        <v>146</v>
       </c>
       <c r="D21" s="116"/>
       <c r="E21" s="116"/>
     </row>
     <row r="22" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="19" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="B22" s="111">
         <v>0.2</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="D22" s="116"/>
       <c r="E22" s="116"/>
     </row>
     <row r="23" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="15" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="B23" s="110">
         <v>0.15</v>
       </c>
-      <c r="C23" s="122" t="s">
-        <v>164</v>
+      <c r="C23" s="123" t="s">
+        <v>150</v>
       </c>
       <c r="D23" s="116"/>
       <c r="E23" s="116"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="117" t="s">
-        <v>165</v>
+      <c r="A25" s="120" t="s">
+        <v>151</v>
       </c>
       <c r="B25" s="116"/>
       <c r="C25" s="116"/>
@@ -4993,72 +4993,72 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="14" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="C26" s="135" t="s">
-        <v>154</v>
+        <v>139</v>
+      </c>
+      <c r="C26" s="122" t="s">
+        <v>140</v>
       </c>
       <c r="D26" s="116"/>
       <c r="E26" s="118"/>
     </row>
     <row r="27" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="15" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="B27" s="110">
         <v>0.25</v>
       </c>
-      <c r="C27" s="122" t="s">
-        <v>167</v>
+      <c r="C27" s="123" t="s">
+        <v>153</v>
       </c>
       <c r="D27" s="116"/>
       <c r="E27" s="116"/>
     </row>
     <row r="28" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="19" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="B28" s="111">
         <v>0.3</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="D28" s="116"/>
       <c r="E28" s="116"/>
     </row>
     <row r="29" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="15" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="B29" s="110">
         <v>0.35</v>
       </c>
-      <c r="C29" s="122" t="s">
-        <v>171</v>
+      <c r="C29" s="123" t="s">
+        <v>157</v>
       </c>
       <c r="D29" s="116"/>
       <c r="E29" s="116"/>
     </row>
     <row r="30" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="19" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="B30" s="111">
         <v>0.1</v>
       </c>
       <c r="C30" s="115" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="D30" s="116"/>
       <c r="E30" s="116"/>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="117" t="s">
-        <v>174</v>
+      <c r="A32" s="120" t="s">
+        <v>160</v>
       </c>
       <c r="B32" s="116"/>
       <c r="C32" s="116"/>
@@ -5067,85 +5067,85 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="14" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="C33" s="135" t="s">
-        <v>154</v>
+        <v>139</v>
+      </c>
+      <c r="C33" s="122" t="s">
+        <v>140</v>
       </c>
       <c r="D33" s="116"/>
       <c r="E33" s="118"/>
     </row>
     <row r="34" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="19" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="B34" s="111">
         <v>0.2</v>
       </c>
       <c r="C34" s="115" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="D34" s="116"/>
       <c r="E34" s="116"/>
     </row>
     <row r="35" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="15" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="B35" s="110">
         <v>0.2</v>
       </c>
-      <c r="C35" s="122" t="s">
-        <v>178</v>
+      <c r="C35" s="123" t="s">
+        <v>164</v>
       </c>
       <c r="D35" s="116"/>
       <c r="E35" s="116"/>
     </row>
     <row r="36" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="19" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="B36" s="111">
         <v>0.15</v>
       </c>
       <c r="C36" s="115" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="D36" s="116"/>
       <c r="E36" s="116"/>
     </row>
     <row r="37" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="15" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="B37" s="110">
         <v>0.2</v>
       </c>
-      <c r="C37" s="122" t="s">
-        <v>182</v>
+      <c r="C37" s="123" t="s">
+        <v>168</v>
       </c>
       <c r="D37" s="116"/>
       <c r="E37" s="116"/>
     </row>
     <row r="38" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="19" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="B38" s="111">
         <v>0.25</v>
       </c>
       <c r="C38" s="115" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="D38" s="116"/>
       <c r="E38" s="116"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="117" t="s">
-        <v>185</v>
+      <c r="A40" s="120" t="s">
+        <v>171</v>
       </c>
       <c r="B40" s="116"/>
       <c r="C40" s="116"/>
@@ -5154,147 +5154,147 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="9" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="23" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="C42" s="24" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="E42" s="26" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="F42" s="27" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="28" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="B43" s="28" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="C43" s="24" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="E43" s="26" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="23" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="C44" s="24" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="E44" s="26" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="F44" s="27" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="28" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="B45" s="28" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="C45" s="24" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="E45" s="26" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="F45" s="27" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="23" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="E46" s="26" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="28" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="B47" s="28" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="C47" s="24" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="E47" s="26" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="F47" s="27" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="117" t="s">
-        <v>222</v>
+      <c r="A49" s="120" t="s">
+        <v>208</v>
       </c>
       <c r="B49" s="116"/>
       <c r="C49" s="116"/>
@@ -5302,8 +5302,8 @@
       <c r="E49" s="118"/>
     </row>
     <row r="50" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="134" t="s">
-        <v>223</v>
+      <c r="A50" s="129" t="s">
+        <v>391</v>
       </c>
       <c r="B50" s="114"/>
       <c r="C50" s="114"/>
@@ -5312,13 +5312,13 @@
     </row>
     <row r="51" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="9" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C51" s="121" t="s">
-        <v>225</v>
+        <v>43</v>
+      </c>
+      <c r="C51" s="117" t="s">
+        <v>210</v>
       </c>
       <c r="D51" s="116"/>
       <c r="E51" s="118"/>
@@ -5328,10 +5328,10 @@
         <v>1</v>
       </c>
       <c r="B52" s="30" t="s">
-        <v>226</v>
-      </c>
-      <c r="C52" s="120" t="s">
-        <v>227</v>
+        <v>211</v>
+      </c>
+      <c r="C52" s="121" t="s">
+        <v>212</v>
       </c>
       <c r="D52" s="116"/>
       <c r="E52" s="116"/>
@@ -5341,10 +5341,10 @@
         <v>2</v>
       </c>
       <c r="B53" s="32" t="s">
-        <v>228</v>
-      </c>
-      <c r="C53" s="127" t="s">
-        <v>229</v>
+        <v>213</v>
+      </c>
+      <c r="C53" s="119" t="s">
+        <v>214</v>
       </c>
       <c r="D53" s="116"/>
       <c r="E53" s="116"/>
@@ -5354,10 +5354,10 @@
         <v>3</v>
       </c>
       <c r="B54" s="30" t="s">
-        <v>230</v>
-      </c>
-      <c r="C54" s="120" t="s">
-        <v>231</v>
+        <v>215</v>
+      </c>
+      <c r="C54" s="121" t="s">
+        <v>216</v>
       </c>
       <c r="D54" s="116"/>
       <c r="E54" s="116"/>
@@ -5367,10 +5367,10 @@
         <v>4</v>
       </c>
       <c r="B55" s="32" t="s">
-        <v>232</v>
-      </c>
-      <c r="C55" s="127" t="s">
-        <v>233</v>
+        <v>217</v>
+      </c>
+      <c r="C55" s="119" t="s">
+        <v>218</v>
       </c>
       <c r="D55" s="116"/>
       <c r="E55" s="116"/>
@@ -5380,17 +5380,17 @@
         <v>5</v>
       </c>
       <c r="B56" s="30" t="s">
-        <v>234</v>
-      </c>
-      <c r="C56" s="120" t="s">
-        <v>235</v>
+        <v>219</v>
+      </c>
+      <c r="C56" s="121" t="s">
+        <v>220</v>
       </c>
       <c r="D56" s="116"/>
       <c r="E56" s="116"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="117" t="s">
-        <v>236</v>
+      <c r="A58" s="120" t="s">
+        <v>221</v>
       </c>
       <c r="B58" s="116"/>
       <c r="C58" s="116"/>
@@ -5399,13 +5399,13 @@
     </row>
     <row r="59" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="9" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C59" s="121" t="s">
-        <v>238</v>
+        <v>43</v>
+      </c>
+      <c r="C59" s="117" t="s">
+        <v>223</v>
       </c>
       <c r="D59" s="116"/>
       <c r="E59" s="118"/>
@@ -5415,10 +5415,10 @@
         <v>1</v>
       </c>
       <c r="B60" s="30" t="s">
-        <v>239</v>
-      </c>
-      <c r="C60" s="120" t="s">
-        <v>240</v>
+        <v>224</v>
+      </c>
+      <c r="C60" s="121" t="s">
+        <v>225</v>
       </c>
       <c r="D60" s="116"/>
       <c r="E60" s="116"/>
@@ -5428,10 +5428,10 @@
         <v>2</v>
       </c>
       <c r="B61" s="32" t="s">
-        <v>241</v>
-      </c>
-      <c r="C61" s="127" t="s">
-        <v>242</v>
+        <v>226</v>
+      </c>
+      <c r="C61" s="119" t="s">
+        <v>227</v>
       </c>
       <c r="D61" s="116"/>
       <c r="E61" s="116"/>
@@ -5441,10 +5441,10 @@
         <v>3</v>
       </c>
       <c r="B62" s="30" t="s">
-        <v>243</v>
-      </c>
-      <c r="C62" s="120" t="s">
-        <v>244</v>
+        <v>228</v>
+      </c>
+      <c r="C62" s="121" t="s">
+        <v>229</v>
       </c>
       <c r="D62" s="116"/>
       <c r="E62" s="116"/>
@@ -5454,10 +5454,10 @@
         <v>4</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>245</v>
-      </c>
-      <c r="C63" s="127" t="s">
-        <v>246</v>
+        <v>230</v>
+      </c>
+      <c r="C63" s="119" t="s">
+        <v>231</v>
       </c>
       <c r="D63" s="116"/>
       <c r="E63" s="116"/>
@@ -5467,17 +5467,17 @@
         <v>5</v>
       </c>
       <c r="B64" s="30" t="s">
-        <v>247</v>
-      </c>
-      <c r="C64" s="120" t="s">
-        <v>248</v>
+        <v>232</v>
+      </c>
+      <c r="C64" s="121" t="s">
+        <v>233</v>
       </c>
       <c r="D64" s="116"/>
       <c r="E64" s="116"/>
     </row>
     <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="117" t="s">
-        <v>249</v>
+      <c r="A66" s="120" t="s">
+        <v>392</v>
       </c>
       <c r="B66" s="116"/>
       <c r="C66" s="116"/>
@@ -5485,8 +5485,8 @@
       <c r="E66" s="118"/>
     </row>
     <row r="67" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" s="136" t="s">
-        <v>250</v>
+      <c r="A67" s="130" t="s">
+        <v>234</v>
       </c>
       <c r="B67" s="114"/>
       <c r="C67" s="114"/>
@@ -5495,85 +5495,85 @@
     </row>
     <row r="68" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="9" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="C68" s="121" t="s">
-        <v>253</v>
+        <v>236</v>
+      </c>
+      <c r="C68" s="117" t="s">
+        <v>237</v>
       </c>
       <c r="D68" s="116"/>
       <c r="E68" s="118"/>
     </row>
     <row r="69" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="36" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B69" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="C69" s="125" t="s">
-        <v>255</v>
+        <v>238</v>
+      </c>
+      <c r="C69" s="124" t="s">
+        <v>239</v>
       </c>
       <c r="D69" s="116"/>
       <c r="E69" s="116"/>
     </row>
     <row r="70" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="38" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B70" s="37" t="s">
-        <v>256</v>
-      </c>
-      <c r="C70" s="125" t="s">
-        <v>257</v>
+        <v>240</v>
+      </c>
+      <c r="C70" s="124" t="s">
+        <v>241</v>
       </c>
       <c r="D70" s="116"/>
       <c r="E70" s="116"/>
     </row>
     <row r="71" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="39" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B71" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="C71" s="125" t="s">
-        <v>259</v>
+        <v>242</v>
+      </c>
+      <c r="C71" s="124" t="s">
+        <v>243</v>
       </c>
       <c r="D71" s="116"/>
       <c r="E71" s="116"/>
     </row>
     <row r="72" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="40" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="C72" s="125" t="s">
-        <v>261</v>
+        <v>244</v>
+      </c>
+      <c r="C72" s="124" t="s">
+        <v>245</v>
       </c>
       <c r="D72" s="116"/>
       <c r="E72" s="116"/>
     </row>
     <row r="73" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="41" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B73" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="C73" s="125" t="s">
-        <v>263</v>
+        <v>246</v>
+      </c>
+      <c r="C73" s="124" t="s">
+        <v>247</v>
       </c>
       <c r="D73" s="116"/>
       <c r="E73" s="116"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="117" t="s">
-        <v>264</v>
+      <c r="A75" s="120" t="s">
+        <v>248</v>
       </c>
       <c r="B75" s="116"/>
       <c r="C75" s="116"/>
@@ -5582,46 +5582,46 @@
     </row>
     <row r="76" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="19" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="B76" s="111">
         <v>0.4</v>
       </c>
-      <c r="C76" s="120" t="s">
-        <v>266</v>
+      <c r="C76" s="121" t="s">
+        <v>250</v>
       </c>
       <c r="D76" s="116"/>
       <c r="E76" s="116"/>
     </row>
     <row r="77" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="15" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="B77" s="110">
         <v>0.4</v>
       </c>
-      <c r="C77" s="127" t="s">
-        <v>268</v>
+      <c r="C77" s="119" t="s">
+        <v>252</v>
       </c>
       <c r="D77" s="116"/>
       <c r="E77" s="116"/>
     </row>
     <row r="78" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="19" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="B78" s="111">
         <v>0.2</v>
       </c>
-      <c r="C78" s="120" t="s">
-        <v>270</v>
+      <c r="C78" s="121" t="s">
+        <v>388</v>
       </c>
       <c r="D78" s="116"/>
       <c r="E78" s="116"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="123" t="s">
-        <v>271</v>
+      <c r="A79" s="136" t="s">
+        <v>254</v>
       </c>
       <c r="B79" s="114"/>
       <c r="C79" s="114"/>
@@ -5630,7 +5630,7 @@
     </row>
     <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="42" t="s">
-        <v>272</v>
+        <v>393</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -5638,7 +5638,7 @@
     <row r="84" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="86" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="43" t="s">
-        <v>273</v>
+        <v>255</v>
       </c>
       <c r="B86" s="44"/>
       <c r="C86" s="44"/>
@@ -5647,8 +5647,8 @@
       <c r="F86" s="44"/>
     </row>
     <row r="87" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="126" t="s">
-        <v>274</v>
+      <c r="A87" s="131" t="s">
+        <v>394</v>
       </c>
       <c r="B87" s="114"/>
       <c r="C87" s="114"/>
@@ -5658,22 +5658,22 @@
     </row>
     <row r="89" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="12" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="D89" s="12" t="s">
-        <v>278</v>
+        <v>259</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="F89" s="12" t="s">
-        <v>279</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5690,10 +5690,10 @@
         <v>1</v>
       </c>
       <c r="E90" s="46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F90" s="45" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5710,10 +5710,10 @@
         <v>2</v>
       </c>
       <c r="E91" s="46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F91" s="45" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5730,10 +5730,10 @@
         <v>3</v>
       </c>
       <c r="E92" s="46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F92" s="45" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5750,10 +5750,10 @@
         <v>4</v>
       </c>
       <c r="E93" s="46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F93" s="45" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5770,10 +5770,10 @@
         <v>5</v>
       </c>
       <c r="E94" s="46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F94" s="45" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5790,10 +5790,10 @@
         <v>6</v>
       </c>
       <c r="E95" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F95" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5810,10 +5810,10 @@
         <v>7</v>
       </c>
       <c r="E96" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F96" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5830,10 +5830,10 @@
         <v>8</v>
       </c>
       <c r="E97" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F97" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5850,10 +5850,10 @@
         <v>9</v>
       </c>
       <c r="E98" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5870,10 +5870,10 @@
         <v>10</v>
       </c>
       <c r="E99" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F99" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5890,10 +5890,10 @@
         <v>11</v>
       </c>
       <c r="E100" s="47" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F100" s="45" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5910,10 +5910,10 @@
         <v>12</v>
       </c>
       <c r="E101" s="48" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F101" s="45" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5930,10 +5930,10 @@
         <v>13</v>
       </c>
       <c r="E102" s="48" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F102" s="45" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5950,10 +5950,10 @@
         <v>14</v>
       </c>
       <c r="E103" s="48" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F103" s="45" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5970,10 +5970,10 @@
         <v>15</v>
       </c>
       <c r="E104" s="48" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F104" s="45" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5990,10 +5990,10 @@
         <v>16</v>
       </c>
       <c r="E105" s="49" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F105" s="45" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6010,10 +6010,10 @@
         <v>17</v>
       </c>
       <c r="E106" s="49" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6030,10 +6030,10 @@
         <v>18</v>
       </c>
       <c r="E107" s="49" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F107" s="45" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6050,10 +6050,10 @@
         <v>19</v>
       </c>
       <c r="E108" s="49" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F108" s="45" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6070,10 +6070,10 @@
         <v>20</v>
       </c>
       <c r="E109" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F109" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6090,10 +6090,10 @@
         <v>21</v>
       </c>
       <c r="E110" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F110" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6110,10 +6110,10 @@
         <v>22</v>
       </c>
       <c r="E111" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F111" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6130,10 +6130,10 @@
         <v>23</v>
       </c>
       <c r="E112" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F112" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6150,10 +6150,10 @@
         <v>24</v>
       </c>
       <c r="E113" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F113" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6170,15 +6170,15 @@
         <v>25</v>
       </c>
       <c r="E114" s="50" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F114" s="45" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
     </row>
     <row r="116" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" s="126" t="s">
-        <v>285</v>
+      <c r="A116" s="131" t="s">
+        <v>395</v>
       </c>
       <c r="B116" s="114"/>
       <c r="C116" s="114"/>
@@ -6188,7 +6188,7 @@
     </row>
     <row r="118" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="43" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
       <c r="B118" s="44"/>
       <c r="C118" s="44"/>
@@ -6197,8 +6197,8 @@
       <c r="F118" s="44"/>
     </row>
     <row r="119" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" s="126" t="s">
-        <v>287</v>
+      <c r="A119" s="131" t="s">
+        <v>267</v>
       </c>
       <c r="B119" s="114"/>
       <c r="C119" s="114"/>
@@ -6208,53 +6208,53 @@
     </row>
     <row r="121" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="51" t="s">
-        <v>288</v>
-      </c>
-      <c r="B121" s="129" t="s">
-        <v>289</v>
+        <v>268</v>
+      </c>
+      <c r="B121" s="133" t="s">
+        <v>269</v>
       </c>
       <c r="C121" s="114"/>
       <c r="D121" s="114"/>
       <c r="E121" s="51" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="52" t="s">
-        <v>100</v>
-      </c>
-      <c r="B122" s="130" t="s">
-        <v>291</v>
-      </c>
-      <c r="C122" s="131"/>
-      <c r="D122" s="132"/>
+        <v>90</v>
+      </c>
+      <c r="B122" s="126" t="s">
+        <v>271</v>
+      </c>
+      <c r="C122" s="127"/>
+      <c r="D122" s="128"/>
       <c r="E122" s="53"/>
     </row>
     <row r="123" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="54" t="s">
-        <v>101</v>
-      </c>
-      <c r="B123" s="130" t="s">
-        <v>292</v>
-      </c>
-      <c r="C123" s="131"/>
-      <c r="D123" s="132"/>
+        <v>91</v>
+      </c>
+      <c r="B123" s="126" t="s">
+        <v>272</v>
+      </c>
+      <c r="C123" s="127"/>
+      <c r="D123" s="128"/>
       <c r="E123" s="53"/>
     </row>
     <row r="124" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="55" t="s">
-        <v>102</v>
-      </c>
-      <c r="B124" s="130" t="s">
-        <v>293</v>
-      </c>
-      <c r="C124" s="131"/>
-      <c r="D124" s="132"/>
+        <v>92</v>
+      </c>
+      <c r="B124" s="126" t="s">
+        <v>273</v>
+      </c>
+      <c r="C124" s="127"/>
+      <c r="D124" s="128"/>
       <c r="E124" s="53"/>
     </row>
     <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A127" s="93" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="B127" s="94"/>
       <c r="C127" s="94"/>
@@ -6263,8 +6263,8 @@
       <c r="F127" s="94"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A129" s="124" t="s">
-        <v>295</v>
+      <c r="A129" s="137" t="s">
+        <v>275</v>
       </c>
       <c r="B129" s="114"/>
       <c r="C129" s="114"/>
@@ -6274,87 +6274,87 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A130" s="95" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="B130" s="95" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="C130" s="95" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="D130" s="95" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="E130" s="95" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="F130" s="95" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="96" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="B131" s="96" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="C131" s="96" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="D131" s="96" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="E131" s="96" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="F131" s="96" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="96" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="B132" s="96" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="C132" s="96" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="D132" s="96" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="E132" s="96" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="F132" s="96" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="96" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="B133" s="96" t="s">
-        <v>311</v>
+        <v>389</v>
       </c>
       <c r="C133" s="96" t="s">
-        <v>312</v>
+        <v>291</v>
       </c>
       <c r="D133" s="96" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="E133" s="96" t="s">
-        <v>313</v>
+        <v>292</v>
       </c>
       <c r="F133" s="96" t="s">
-        <v>314</v>
+        <v>293</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A136" s="119" t="s">
-        <v>315</v>
+      <c r="A136" s="135" t="s">
+        <v>294</v>
       </c>
       <c r="B136" s="114"/>
       <c r="C136" s="114"/>
@@ -6364,7 +6364,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A139" s="93" t="s">
-        <v>316</v>
+        <v>396</v>
       </c>
       <c r="B139" s="94"/>
       <c r="C139" s="94"/>
@@ -6373,8 +6373,8 @@
       <c r="F139" s="94"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A141" s="128" t="s">
-        <v>317</v>
+      <c r="A141" s="132" t="s">
+        <v>397</v>
       </c>
       <c r="B141" s="114"/>
       <c r="C141" s="114"/>
@@ -6384,72 +6384,119 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A143" s="95" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="B143" s="95" t="s">
-        <v>318</v>
+        <v>295</v>
       </c>
       <c r="C143" s="95" t="s">
-        <v>319</v>
+        <v>296</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A144" s="97" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B144" s="98" t="s">
-        <v>320</v>
+        <v>297</v>
       </c>
       <c r="C144" s="98" t="s">
-        <v>321</v>
+        <v>298</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A145" s="99" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B145" s="98" t="s">
-        <v>322</v>
+        <v>299</v>
       </c>
       <c r="C145" s="98" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A146" s="100" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B146" s="98" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
       <c r="C146" s="98" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="101" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B147" s="98" t="s">
-        <v>326</v>
+        <v>303</v>
       </c>
       <c r="C147" s="98" t="s">
-        <v>327</v>
+        <v>304</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A148" s="102" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B148" s="98" t="s">
-        <v>328</v>
+        <v>305</v>
       </c>
       <c r="C148" s="98" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A136:F136"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="A129:F129"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="B122:D122"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B123:D123"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A67:E67"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C68:E68"/>
@@ -6466,53 +6513,6 @@
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="C64:E64"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B123:D123"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="A141:F141"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="B121:D121"/>
-    <mergeCell ref="B122:D122"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A87:F87"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A136:F136"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="A129:F129"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C71:E71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6543,12 +6543,12 @@
   <sheetData>
     <row r="2" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="C2" s="13" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="133" t="s">
-        <v>331</v>
+      <c r="C3" s="125" t="s">
+        <v>308</v>
       </c>
       <c r="D3" s="114"/>
       <c r="E3" s="114"/>
@@ -6557,21 +6557,21 @@
     </row>
     <row r="5" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C5" s="56" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
       <c r="D5" s="57" t="s">
-        <v>333</v>
+        <v>310</v>
       </c>
       <c r="E5" s="56" t="s">
-        <v>334</v>
+        <v>311</v>
       </c>
       <c r="F5" s="57" t="s">
-        <v>335</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C7" s="193" t="s">
-        <v>336</v>
+        <v>313</v>
       </c>
       <c r="D7" s="114"/>
       <c r="E7" s="114"/>
@@ -6580,18 +6580,18 @@
     </row>
     <row r="8" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C8" s="58" t="s">
-        <v>337</v>
+        <v>314</v>
       </c>
       <c r="D8" s="59">
         <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>406</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C9" s="58" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
       <c r="D9" s="59">
         <v>100</v>
@@ -6599,7 +6599,7 @@
     </row>
     <row r="10" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C10" s="58" t="s">
-        <v>339</v>
+        <v>316</v>
       </c>
       <c r="D10" s="59">
         <v>100</v>
@@ -6607,7 +6607,7 @@
     </row>
     <row r="11" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C11" s="56" t="s">
-        <v>340</v>
+        <v>317</v>
       </c>
       <c r="D11" s="60">
         <f>D9/D10</f>
@@ -6616,7 +6616,7 @@
     </row>
     <row r="12" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C12" s="56" t="s">
-        <v>341</v>
+        <v>318</v>
       </c>
       <c r="D12" s="61">
         <f>D9-D10</f>
@@ -6625,7 +6625,7 @@
     </row>
     <row r="13" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C13" s="56" t="s">
-        <v>342</v>
+        <v>319</v>
       </c>
       <c r="D13" s="60">
         <f>D9/D8</f>
@@ -6634,7 +6634,7 @@
     </row>
     <row r="14" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C14" s="56" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
       <c r="D14" s="61">
         <f>D9-D8</f>
@@ -6643,7 +6643,7 @@
     </row>
     <row r="16" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C16" s="193" t="s">
-        <v>344</v>
+        <v>321</v>
       </c>
       <c r="D16" s="114"/>
       <c r="E16" s="114"/>
@@ -6652,7 +6652,7 @@
     </row>
     <row r="17" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C17" s="58" t="s">
-        <v>345</v>
+        <v>322</v>
       </c>
       <c r="D17" s="62">
         <v>0.1</v>
@@ -6660,18 +6660,18 @@
     </row>
     <row r="18" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C18" s="58" t="s">
-        <v>346</v>
+        <v>323</v>
       </c>
       <c r="D18" s="62">
         <v>0.05</v>
       </c>
       <c r="E18" t="s">
-        <v>403</v>
+        <v>379</v>
       </c>
     </row>
     <row r="19" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C19" s="58" t="s">
-        <v>347</v>
+        <v>324</v>
       </c>
       <c r="D19" s="62">
         <v>0.04</v>
@@ -6679,7 +6679,7 @@
     </row>
     <row r="20" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C20" s="58" t="s">
-        <v>348</v>
+        <v>325</v>
       </c>
       <c r="D20" s="62">
         <v>0.06</v>
@@ -6687,7 +6687,7 @@
     </row>
     <row r="21" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C21" s="58" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="D21" s="62">
         <v>0.08</v>
@@ -6695,7 +6695,7 @@
     </row>
     <row r="22" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C22" s="56" t="s">
-        <v>350</v>
+        <v>327</v>
       </c>
       <c r="D22" s="63">
         <f>(D17*0.25+D18*0.2+D19*0.2+D20*0.2+D21*0.15)</f>
@@ -6704,7 +6704,7 @@
     </row>
     <row r="24" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C24" s="193" t="s">
-        <v>351</v>
+        <v>328</v>
       </c>
       <c r="D24" s="114"/>
       <c r="E24" s="114"/>
@@ -6713,82 +6713,82 @@
     </row>
     <row r="25" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C25" s="58" t="s">
-        <v>352</v>
+        <v>329</v>
       </c>
       <c r="D25" s="62">
         <v>0.88</v>
       </c>
       <c r="F25" t="s">
-        <v>337</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C26" s="58" t="s">
-        <v>353</v>
+        <v>330</v>
       </c>
       <c r="D26" s="62">
         <v>0.73</v>
       </c>
       <c r="F26" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C27" s="58" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="D27" s="62">
         <v>0.82</v>
       </c>
       <c r="F27" t="s">
-        <v>339</v>
+        <v>316</v>
       </c>
     </row>
     <row r="28" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C28" s="58" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="D28" s="62">
         <v>0.42</v>
       </c>
       <c r="E28" t="s">
-        <v>405</v>
+        <v>381</v>
       </c>
       <c r="F28" t="s">
-        <v>340</v>
+        <v>317</v>
       </c>
     </row>
     <row r="29" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C29" s="56" t="s">
-        <v>356</v>
+        <v>333</v>
       </c>
       <c r="D29" s="63">
         <f>(D25*0.25+D26*0.3+D27*0.35+D28*0.1)</f>
         <v>0.76800000000000002</v>
       </c>
       <c r="F29" t="s">
-        <v>341</v>
+        <v>318</v>
       </c>
     </row>
     <row r="30" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C30" s="58" t="s">
-        <v>357</v>
+        <v>334</v>
       </c>
       <c r="D30" s="62">
         <v>5.8000000000000003E-2</v>
       </c>
       <c r="F30" t="s">
-        <v>342</v>
+        <v>319</v>
       </c>
     </row>
     <row r="31" spans="3:7" x14ac:dyDescent="0.45">
       <c r="F31" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
     </row>
     <row r="32" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C32" s="193" t="s">
-        <v>358</v>
+        <v>335</v>
       </c>
       <c r="D32" s="114"/>
       <c r="E32" s="114"/>
@@ -6797,7 +6797,7 @@
     </row>
     <row r="33" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C33" s="58" t="s">
-        <v>359</v>
+        <v>336</v>
       </c>
       <c r="D33" s="62">
         <v>0.6</v>
@@ -6805,7 +6805,7 @@
     </row>
     <row r="34" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C34" s="58" t="s">
-        <v>360</v>
+        <v>337</v>
       </c>
       <c r="D34" s="62">
         <v>0.6</v>
@@ -6813,7 +6813,7 @@
     </row>
     <row r="35" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C35" s="58" t="s">
-        <v>361</v>
+        <v>338</v>
       </c>
       <c r="D35" s="62">
         <v>0.8</v>
@@ -6821,7 +6821,7 @@
     </row>
     <row r="36" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C36" s="58" t="s">
-        <v>362</v>
+        <v>339</v>
       </c>
       <c r="D36" s="62">
         <v>0.8</v>
@@ -6829,21 +6829,21 @@
     </row>
     <row r="37" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C37" s="58" t="s">
-        <v>363</v>
+        <v>340</v>
       </c>
       <c r="D37" s="62">
         <v>0.4</v>
       </c>
       <c r="E37" t="s">
-        <v>404</v>
+        <v>380</v>
       </c>
       <c r="F37" t="s">
-        <v>407</v>
+        <v>383</v>
       </c>
     </row>
     <row r="38" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C38" s="56" t="s">
-        <v>364</v>
+        <v>341</v>
       </c>
       <c r="D38" s="63">
         <f>(D33*0.2+D34*0.2+D35*0.15+D36*0.2+D37*0.25)</f>
@@ -6852,7 +6852,7 @@
     </row>
     <row r="40" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C40" s="193" t="s">
-        <v>365</v>
+        <v>342</v>
       </c>
       <c r="D40" s="114"/>
       <c r="E40" s="114"/>
@@ -6861,7 +6861,7 @@
     </row>
     <row r="41" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C41" s="58" t="s">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="D41" s="108">
         <f>D22*100</f>
@@ -6870,7 +6870,7 @@
     </row>
     <row r="42" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C42" s="58" t="s">
-        <v>367</v>
+        <v>344</v>
       </c>
       <c r="D42" s="108">
         <f>D29*100</f>
@@ -6879,7 +6879,7 @@
     </row>
     <row r="43" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C43" s="58" t="s">
-        <v>368</v>
+        <v>345</v>
       </c>
       <c r="D43" s="108">
         <f>D38*100</f>
@@ -6888,7 +6888,7 @@
     </row>
     <row r="44" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C44" s="56" t="s">
-        <v>369</v>
+        <v>346</v>
       </c>
       <c r="D44" s="109">
         <f>(D41*0.4)+(D42*0.4)+(D43*0.2)</f>
@@ -6897,7 +6897,7 @@
     </row>
     <row r="45" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C45" s="56" t="s">
-        <v>370</v>
+        <v>347</v>
       </c>
       <c r="D45" s="65" t="str">
         <f>IF(D44&lt;=20,"Low",IF(D44&lt;=44,"Low to Moderate",IF(D44&lt;=60,"Moderate",IF(D44&lt;=76,"Moderate to High","High"))))</f>
@@ -6906,7 +6906,7 @@
     </row>
     <row r="47" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C47" s="193" t="s">
-        <v>371</v>
+        <v>398</v>
       </c>
       <c r="D47" s="114"/>
       <c r="E47" s="114"/>
@@ -6915,7 +6915,7 @@
     </row>
     <row r="48" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C48" s="87" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D48" s="66">
         <v>5</v>
@@ -6923,7 +6923,7 @@
     </row>
     <row r="49" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C49" s="88" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="D49" s="66">
         <v>11</v>
@@ -6931,7 +6931,7 @@
     </row>
     <row r="50" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C50" s="89" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D50" s="66">
         <v>18</v>
@@ -6939,7 +6939,7 @@
     </row>
     <row r="51" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C51" s="90" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D51" s="66">
         <v>4</v>
@@ -6947,7 +6947,7 @@
     </row>
     <row r="52" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C52" s="86" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D52" s="66">
         <v>3</v>
@@ -6955,7 +6955,7 @@
     </row>
     <row r="53" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C53" s="91" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D53" s="92">
         <f>SUM(D48:D52)</f>
@@ -6971,7 +6971,7 @@
     </row>
     <row r="55" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C55" s="193" t="s">
-        <v>372</v>
+        <v>348</v>
       </c>
       <c r="D55" s="114"/>
       <c r="E55" s="114"/>
@@ -6980,13 +6980,13 @@
     </row>
     <row r="56" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C56" s="58" t="s">
-        <v>373</v>
+        <v>349</v>
       </c>
       <c r="D56" s="62">
         <v>0.82</v>
       </c>
       <c r="E56" s="58" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="F56" s="66">
         <v>2</v>
@@ -6994,13 +6994,13 @@
     </row>
     <row r="57" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C57" s="58" t="s">
-        <v>374</v>
+        <v>350</v>
       </c>
       <c r="D57" s="62">
         <v>0.18</v>
       </c>
       <c r="E57" s="58" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F57" s="66">
         <v>3</v>
@@ -7008,13 +7008,13 @@
     </row>
     <row r="58" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C58" s="58" t="s">
-        <v>375</v>
+        <v>351</v>
       </c>
       <c r="D58" s="62">
         <v>0.76</v>
       </c>
       <c r="E58" s="58" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="F58" s="66">
         <v>5</v>
@@ -7022,13 +7022,13 @@
     </row>
     <row r="59" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C59" s="58" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="D59" s="66">
         <v>5</v>
       </c>
       <c r="E59" s="58" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F59" s="66">
         <v>4</v>
@@ -7043,7 +7043,7 @@
     </row>
     <row r="61" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C61" s="193" t="s">
-        <v>376</v>
+        <v>352</v>
       </c>
       <c r="D61" s="114"/>
       <c r="E61" s="114"/>
@@ -7052,30 +7052,30 @@
     </row>
     <row r="62" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C62" s="14" t="s">
-        <v>377</v>
+        <v>353</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>378</v>
+        <v>354</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>379</v>
+        <v>355</v>
       </c>
       <c r="F62" s="67" t="s">
-        <v>380</v>
+        <v>356</v>
       </c>
       <c r="G62" s="67" t="s">
-        <v>381</v>
+        <v>357</v>
       </c>
       <c r="H62" s="67" t="s">
-        <v>382</v>
+        <v>358</v>
       </c>
     </row>
     <row r="63" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C63" s="58" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D63" s="68" t="s">
-        <v>383</v>
+        <v>359</v>
       </c>
       <c r="E63" s="66">
         <v>24</v>
@@ -7094,10 +7094,10 @@
     </row>
     <row r="64" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C64" s="58" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="D64" s="68" t="s">
-        <v>384</v>
+        <v>360</v>
       </c>
       <c r="E64" s="62">
         <v>0.73</v>
@@ -7116,10 +7116,10 @@
     </row>
     <row r="65" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C65" s="58" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D65" s="68" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E65" s="64">
         <v>0.94</v>
@@ -7138,10 +7138,10 @@
     </row>
     <row r="66" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C66" s="58" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D66" s="68" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E66" s="62">
         <v>0.75</v>
@@ -7160,10 +7160,10 @@
     </row>
     <row r="67" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C67" s="58" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="D67" s="68" t="s">
-        <v>385</v>
+        <v>361</v>
       </c>
       <c r="E67" s="62">
         <v>0.42</v>
@@ -7182,10 +7182,10 @@
     </row>
     <row r="68" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C68" s="58" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="D68" s="68" t="s">
-        <v>386</v>
+        <v>362</v>
       </c>
       <c r="E68" s="62">
         <v>0.4</v>
@@ -7211,7 +7211,7 @@
     </row>
     <row r="71" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C71" s="193" t="s">
-        <v>387</v>
+        <v>363</v>
       </c>
       <c r="D71" s="114"/>
       <c r="E71" s="114"/>
@@ -7220,41 +7220,41 @@
     </row>
     <row r="72" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C72" s="85" t="s">
-        <v>388</v>
+        <v>364</v>
       </c>
     </row>
     <row r="73" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C73" s="9" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>389</v>
+        <v>365</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>390</v>
+        <v>366</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>391</v>
+        <v>367</v>
       </c>
     </row>
     <row r="74" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C74" s="73" t="s">
-        <v>392</v>
+        <v>368</v>
       </c>
       <c r="D74" s="74" t="s">
-        <v>393</v>
+        <v>369</v>
       </c>
       <c r="E74" s="37" t="s">
-        <v>394</v>
+        <v>370</v>
       </c>
       <c r="F74" s="66">
         <v>4</v>
@@ -7273,13 +7273,13 @@
     </row>
     <row r="75" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C75" s="73" t="s">
-        <v>395</v>
+        <v>371</v>
       </c>
       <c r="D75" s="74" t="s">
-        <v>396</v>
+        <v>372</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>397</v>
+        <v>373</v>
       </c>
       <c r="F75" s="66">
         <v>5</v>
@@ -7298,13 +7298,13 @@
     </row>
     <row r="76" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C76" s="73" t="s">
-        <v>398</v>
+        <v>374</v>
       </c>
       <c r="D76" s="74" t="s">
-        <v>399</v>
+        <v>375</v>
       </c>
       <c r="E76" s="37" t="s">
-        <v>397</v>
+        <v>373</v>
       </c>
       <c r="F76" s="66">
         <v>4</v>
@@ -7323,13 +7323,13 @@
     </row>
     <row r="77" spans="3:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C77" s="73" t="s">
-        <v>400</v>
+        <v>376</v>
       </c>
       <c r="D77" s="74" t="s">
-        <v>401</v>
+        <v>377</v>
       </c>
       <c r="E77" s="37" t="s">
-        <v>402</v>
+        <v>378</v>
       </c>
       <c r="F77" s="66">
         <v>3</v>
@@ -7397,8 +7397,8 @@
       <c r="G2" s="114"/>
     </row>
     <row r="3" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="133" t="s">
-        <v>1</v>
+      <c r="B3" s="125" t="s">
+        <v>400</v>
       </c>
       <c r="C3" s="114"/>
       <c r="D3" s="114"/>
@@ -7408,45 +7408,45 @@
     </row>
     <row r="5" spans="2:26" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="75" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="75" t="s">
+      <c r="D5" s="75" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="75" t="s">
+      <c r="E5" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="75" t="s">
+      <c r="F5" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="75" t="s">
+      <c r="G5" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="75" t="s">
+      <c r="Z5" t="s">
         <v>7</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="6" spans="2:26" ht="73.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="76" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="D6" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78" t="s">
+      <c r="E6" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="F6" s="77" t="s">
+        <v>399</v>
+      </c>
+      <c r="G6" s="77" t="s">
         <v>12</v>
-      </c>
-      <c r="F6" s="77" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="77" t="s">
-        <v>14</v>
       </c>
       <c r="Z6" s="77">
         <f t="shared" ref="Z6:Z15" si="0">IF(D6="","", IF(ISNUMBER(SEARCH("Moderate to High", D6)), 40, IF(ISNUMBER(SEARCH("High", D6)), 50, IF(ISNUMBER(SEARCH("Low to Moderate", D6)), 20, IF(ISNUMBER(SEARCH("Moderate", D6)), 30, 10)))) + (1/ROW()))</f>
@@ -7455,22 +7455,22 @@
     </row>
     <row r="7" spans="2:26" ht="73.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="76" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="77" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="77" t="s">
+      <c r="E7" s="77" t="s">
+        <v>406</v>
+      </c>
+      <c r="F7" s="77" t="s">
+        <v>401</v>
+      </c>
+      <c r="G7" s="77" t="s">
         <v>16</v>
-      </c>
-      <c r="D7" s="79" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="77" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="77" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="77" t="s">
-        <v>20</v>
       </c>
       <c r="Z7" s="77">
         <f t="shared" si="0"/>
@@ -7479,22 +7479,22 @@
     </row>
     <row r="8" spans="2:26" ht="73.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="76" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="77" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="79" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="77" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="77" t="s">
+        <v>402</v>
+      </c>
+      <c r="G8" s="77" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="79" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="77" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="77" t="s">
-        <v>26</v>
       </c>
       <c r="Z8" s="77">
         <f t="shared" si="0"/>
@@ -7503,22 +7503,22 @@
     </row>
     <row r="9" spans="2:26" ht="73.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="76" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C9" s="77" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D9" s="80" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E9" s="77" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F9" s="77" t="s">
-        <v>31</v>
+        <v>403</v>
       </c>
       <c r="G9" s="77" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="Z9" s="77">
         <f t="shared" si="0"/>
@@ -7527,22 +7527,22 @@
     </row>
     <row r="10" spans="2:26" ht="73.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="76" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C10" s="77" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D10" s="80" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E10" s="77" t="s">
-        <v>36</v>
+        <v>407</v>
       </c>
       <c r="F10" s="77" t="s">
-        <v>37</v>
+        <v>404</v>
       </c>
       <c r="G10" s="77" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="Z10" s="77">
         <f t="shared" si="0"/>
@@ -7557,7 +7557,7 @@
     </row>
     <row r="12" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="197" t="s">
-        <v>39</v>
+        <v>405</v>
       </c>
       <c r="C12" s="114"/>
       <c r="D12" s="114"/>
@@ -7601,7 +7601,7 @@
     </row>
     <row r="16" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B16" s="196" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C16" s="114"/>
       <c r="D16" s="114"/>
@@ -7611,14 +7611,14 @@
     </row>
     <row r="17" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="81" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C17" s="82">
         <f>Input_Bulanan!F56</f>
         <v>2</v>
       </c>
       <c r="D17" s="195" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E17" s="116"/>
       <c r="F17" s="116"/>
@@ -7626,14 +7626,14 @@
     </row>
     <row r="18" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B18" s="81" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C18" s="82">
         <f>Input_Bulanan!F57</f>
         <v>3</v>
       </c>
       <c r="D18" s="195" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E18" s="116"/>
       <c r="F18" s="116"/>
@@ -7641,14 +7641,14 @@
     </row>
     <row r="19" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B19" s="81" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C19" s="82">
         <f>Input_Bulanan!F58</f>
         <v>5</v>
       </c>
       <c r="D19" s="195" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E19" s="116"/>
       <c r="F19" s="116"/>
@@ -7656,14 +7656,14 @@
     </row>
     <row r="20" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B20" s="81" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C20" s="82">
         <f>Input_Bulanan!F59</f>
         <v>4</v>
       </c>
       <c r="D20" s="195" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E20" s="116"/>
       <c r="F20" s="116"/>
@@ -7671,7 +7671,7 @@
     </row>
     <row r="22" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B22" s="196" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C22" s="114"/>
       <c r="D22" s="114"/>
@@ -7681,22 +7681,22 @@
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B23" s="11" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Menukar sumbu Likelihood dan Consequence pada Heatmap Excel
</commit_message>
<xml_diff>
--- a/Template_Dashboard.xlsx
+++ b/Template_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365mic-my.sharepoint.com/personal/ipanjez_365mic_onmicrosoft_com/Documents/Learn/Coding/Dashboard Proyek Soda Ash/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{901E0FE3-4737-4F4F-849C-FBD9465FF939}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25C4878D-1B90-4CEB-854D-FFE7585F0910}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -675,28 +675,10 @@
     <t>Supply Readiness Index (SRI)</t>
   </si>
   <si>
-    <t>C=5</t>
-  </si>
-  <si>
-    <t>C=4</t>
-  </si>
-  <si>
     <t>Project Execution Index (PEI)</t>
   </si>
   <si>
-    <t>C=3</t>
-  </si>
-  <si>
-    <t>C=2</t>
-  </si>
-  <si>
     <t>Commercial Readiness Index (CRI)</t>
-  </si>
-  <si>
-    <t>C=1</t>
-  </si>
-  <si>
-    <t>L -&gt;</t>
   </si>
   <si>
     <t>Key Financial &amp; Schedule</t>
@@ -1739,6 +1721,24 @@
   </si>
   <si>
     <t>Membentuk tim percepatan perizinan internal untuk koordinasi harian dengan DLH Kota X dan Dinas PUPR Provinsi Provinsi X guna mempercepat adendum dokumen lingkungan di lahan sengketa.</t>
+  </si>
+  <si>
+    <t>L=5</t>
+  </si>
+  <si>
+    <t>L=4</t>
+  </si>
+  <si>
+    <t>L=3</t>
+  </si>
+  <si>
+    <t>L=2</t>
+  </si>
+  <si>
+    <t>L=1</t>
+  </si>
+  <si>
+    <t>C -&gt;</t>
   </si>
 </sst>
 </file>
@@ -2763,207 +2763,207 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3382,8 +3382,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="182" t="s">
-        <v>384</v>
+      <c r="B1" s="167" t="s">
+        <v>378</v>
       </c>
       <c r="C1" s="116"/>
       <c r="D1" s="116"/>
@@ -3408,7 +3408,7 @@
       <c r="W1" s="118"/>
     </row>
     <row r="2" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="152" t="str">
+      <c r="B2" s="186" t="str">
         <f ca="1">"Reporting Period: "&amp;Input_Bulanan!D5&amp;"   |   Status: "&amp;Input_Bulanan!F5&amp;"   |   Dicetak: "&amp;TEXT(TODAY(),"DD-MM-YYYY")</f>
         <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 18-07-2026</v>
       </c>
@@ -3436,7 +3436,7 @@
     </row>
     <row r="3" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="153" t="s">
+      <c r="B4" s="138" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="116"/>
@@ -3449,7 +3449,7 @@
       <c r="J4" s="116"/>
       <c r="K4" s="116"/>
       <c r="L4" s="118"/>
-      <c r="M4" s="153" t="s">
+      <c r="M4" s="138" t="s">
         <v>48</v>
       </c>
       <c r="N4" s="116"/>
@@ -3464,14 +3464,14 @@
       <c r="W4" s="118"/>
     </row>
     <row r="5" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="162" t="s">
+      <c r="B5" s="152" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="116"/>
       <c r="D5" s="116"/>
       <c r="E5" s="116"/>
       <c r="F5" s="118"/>
-      <c r="G5" s="162" t="s">
+      <c r="G5" s="152" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="116"/>
@@ -3479,14 +3479,14 @@
       <c r="J5" s="116"/>
       <c r="K5" s="116"/>
       <c r="L5" s="118"/>
-      <c r="M5" s="162" t="s">
+      <c r="M5" s="152" t="s">
         <v>51</v>
       </c>
       <c r="N5" s="116"/>
       <c r="O5" s="116"/>
       <c r="P5" s="116"/>
       <c r="Q5" s="118"/>
-      <c r="R5" s="147" t="s">
+      <c r="R5" s="188" t="s">
         <v>52</v>
       </c>
       <c r="S5" s="116"/>
@@ -3496,51 +3496,51 @@
       <c r="W5" s="118"/>
     </row>
     <row r="6" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="192">
+      <c r="B6" s="154">
         <f>((IF(Input_Bulanan!D11&gt;=1,100,Input_Bulanan!D11*100)*0.2)+(IF(Input_Bulanan!D13&gt;=1,100,Input_Bulanan!D13*100)*0.2)+(Input_Bulanan!D22*100*0.2)+(Input_Bulanan!D29*100*0.2)+(Input_Bulanan!D38*100*0.2))/100</f>
         <v>0.69100000000000006</v>
       </c>
-      <c r="C6" s="156"/>
-      <c r="D6" s="156"/>
-      <c r="E6" s="156"/>
-      <c r="F6" s="142"/>
-      <c r="G6" s="160" t="s">
+      <c r="C6" s="142"/>
+      <c r="D6" s="142"/>
+      <c r="E6" s="142"/>
+      <c r="F6" s="143"/>
+      <c r="G6" s="173" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="156"/>
-      <c r="I6" s="156"/>
-      <c r="J6" s="156"/>
-      <c r="K6" s="141">
+      <c r="H6" s="142"/>
+      <c r="I6" s="142"/>
+      <c r="J6" s="142"/>
+      <c r="K6" s="148">
         <f>Input_Bulanan!D22</f>
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="L6" s="142"/>
-      <c r="M6" s="155" t="str">
+      <c r="L6" s="143"/>
+      <c r="M6" s="187" t="str">
         <f>Input_Bulanan!D45</f>
         <v>Moderate</v>
       </c>
-      <c r="N6" s="156"/>
-      <c r="O6" s="156"/>
-      <c r="P6" s="156"/>
-      <c r="Q6" s="142"/>
+      <c r="N6" s="142"/>
+      <c r="O6" s="142"/>
+      <c r="P6" s="142"/>
+      <c r="Q6" s="143"/>
       <c r="R6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="S6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <v>402</v>
+      </c>
+      <c r="S6" s="5" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="T6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+      <c r="T6" s="3" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="U6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+      <c r="U6" s="4" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="V6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
-        <v>C1</v>
+        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <v/>
       </c>
       <c r="W6" s="2" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
@@ -3548,35 +3548,35 @@
       </c>
     </row>
     <row r="7" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="157"/>
+      <c r="B7" s="155"/>
       <c r="C7" s="114"/>
       <c r="D7" s="114"/>
       <c r="E7" s="114"/>
-      <c r="F7" s="158"/>
-      <c r="G7" s="159"/>
-      <c r="H7" s="143"/>
-      <c r="I7" s="143"/>
-      <c r="J7" s="143"/>
-      <c r="K7" s="143"/>
-      <c r="L7" s="144"/>
-      <c r="M7" s="157"/>
+      <c r="F7" s="156"/>
+      <c r="G7" s="144"/>
+      <c r="H7" s="145"/>
+      <c r="I7" s="145"/>
+      <c r="J7" s="145"/>
+      <c r="K7" s="145"/>
+      <c r="L7" s="146"/>
+      <c r="M7" s="155"/>
       <c r="N7" s="114"/>
       <c r="O7" s="114"/>
       <c r="P7" s="114"/>
-      <c r="Q7" s="158"/>
+      <c r="Q7" s="156"/>
       <c r="R7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="S7" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <v>403</v>
+      </c>
+      <c r="S7" s="6" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="T7" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+      <c r="T7" s="5" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="U7" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+      <c r="U7" s="3" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="V7" s="4" t="str">
@@ -3584,78 +3584,78 @@
         <v>C3</v>
       </c>
       <c r="W7" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
-        <v/>
+        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <v>C1</v>
       </c>
     </row>
     <row r="8" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="157"/>
+      <c r="B8" s="155"/>
       <c r="C8" s="114"/>
       <c r="D8" s="114"/>
       <c r="E8" s="114"/>
-      <c r="F8" s="158"/>
-      <c r="G8" s="160" t="s">
-        <v>56</v>
-      </c>
-      <c r="H8" s="156"/>
-      <c r="I8" s="156"/>
-      <c r="J8" s="156"/>
-      <c r="K8" s="141">
+      <c r="F8" s="156"/>
+      <c r="G8" s="173" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="142"/>
+      <c r="I8" s="142"/>
+      <c r="J8" s="142"/>
+      <c r="K8" s="148">
         <f>Input_Bulanan!D29</f>
         <v>0.76800000000000002</v>
       </c>
-      <c r="L8" s="142"/>
-      <c r="M8" s="157"/>
+      <c r="L8" s="143"/>
+      <c r="M8" s="155"/>
       <c r="N8" s="114"/>
       <c r="O8" s="114"/>
       <c r="P8" s="114"/>
-      <c r="Q8" s="158"/>
+      <c r="Q8" s="156"/>
       <c r="R8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="S8" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <v>404</v>
+      </c>
+      <c r="S8" s="6" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="T8" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="U8" s="3" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
         <v>C4</v>
       </c>
-      <c r="V8" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+      <c r="V8" s="4" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="W8" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+      <c r="W8" s="2" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="159"/>
-      <c r="C9" s="143"/>
-      <c r="D9" s="143"/>
-      <c r="E9" s="143"/>
-      <c r="F9" s="144"/>
-      <c r="G9" s="159"/>
-      <c r="H9" s="143"/>
-      <c r="I9" s="143"/>
-      <c r="J9" s="143"/>
-      <c r="K9" s="143"/>
-      <c r="L9" s="144"/>
-      <c r="M9" s="159"/>
-      <c r="N9" s="143"/>
-      <c r="O9" s="143"/>
-      <c r="P9" s="143"/>
-      <c r="Q9" s="144"/>
+      <c r="B9" s="144"/>
+      <c r="C9" s="145"/>
+      <c r="D9" s="145"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="146"/>
+      <c r="G9" s="144"/>
+      <c r="H9" s="145"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="146"/>
+      <c r="M9" s="144"/>
+      <c r="N9" s="145"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="145"/>
+      <c r="Q9" s="146"/>
       <c r="R9" s="1" t="s">
-        <v>58</v>
+        <v>405</v>
       </c>
       <c r="S9" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="T9" s="5" t="str">
@@ -3663,89 +3663,89 @@
         <v/>
       </c>
       <c r="U9" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="V9" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+      <c r="V9" s="4" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="W9" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+      <c r="W9" s="2" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="191" t="str">
+      <c r="B10" s="141" t="str">
         <f>IF(B6&gt;=0.9,"HIJAU - SEHAT",IF(B6&gt;=0.75,"KUNING - PANTAU",IF(B6&gt;=0.6,"ORANYE - WASPADA","MERAH - KRITIS")))</f>
         <v>ORANYE - WASPADA</v>
       </c>
-      <c r="C10" s="156"/>
-      <c r="D10" s="156"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="142"/>
-      <c r="G10" s="160" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="156"/>
-      <c r="I10" s="156"/>
-      <c r="J10" s="156"/>
-      <c r="K10" s="141">
+      <c r="C10" s="142"/>
+      <c r="D10" s="142"/>
+      <c r="E10" s="142"/>
+      <c r="F10" s="143"/>
+      <c r="G10" s="173" t="s">
+        <v>55</v>
+      </c>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="148">
         <f>Input_Bulanan!D38</f>
         <v>0.62</v>
       </c>
-      <c r="L10" s="142"/>
-      <c r="M10" s="168" t="str">
+      <c r="L10" s="143"/>
+      <c r="M10" s="175" t="str">
         <f>"Skor Komposit: "&amp;TEXT(Input_Bulanan!D44,"0,00")&amp;" / 100"</f>
         <v>Skor Komposit: 45,80 / 100</v>
       </c>
-      <c r="N10" s="156"/>
-      <c r="O10" s="156"/>
-      <c r="P10" s="156"/>
-      <c r="Q10" s="142"/>
+      <c r="N10" s="142"/>
+      <c r="O10" s="142"/>
+      <c r="P10" s="142"/>
+      <c r="Q10" s="143"/>
       <c r="R10" s="1" t="s">
-        <v>60</v>
+        <v>406</v>
       </c>
       <c r="S10" s="6" t="str">
         <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
       <c r="T10" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="U10" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+      <c r="U10" s="5" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="V10" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+      <c r="V10" s="3" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
-      <c r="W10" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+      <c r="W10" s="2" t="str">
+        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="2:23" ht="12" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="159"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="143"/>
-      <c r="E11" s="143"/>
-      <c r="F11" s="144"/>
-      <c r="G11" s="159"/>
-      <c r="H11" s="143"/>
-      <c r="I11" s="143"/>
-      <c r="J11" s="143"/>
-      <c r="K11" s="143"/>
-      <c r="L11" s="144"/>
-      <c r="M11" s="159"/>
-      <c r="N11" s="143"/>
-      <c r="O11" s="143"/>
-      <c r="P11" s="143"/>
-      <c r="Q11" s="144"/>
+      <c r="B11" s="144"/>
+      <c r="C11" s="145"/>
+      <c r="D11" s="145"/>
+      <c r="E11" s="145"/>
+      <c r="F11" s="146"/>
+      <c r="G11" s="144"/>
+      <c r="H11" s="145"/>
+      <c r="I11" s="145"/>
+      <c r="J11" s="145"/>
+      <c r="K11" s="145"/>
+      <c r="L11" s="146"/>
+      <c r="M11" s="144"/>
+      <c r="N11" s="145"/>
+      <c r="O11" s="145"/>
+      <c r="P11" s="145"/>
+      <c r="Q11" s="146"/>
       <c r="R11" s="7" t="s">
-        <v>61</v>
+        <v>407</v>
       </c>
       <c r="S11" s="8">
         <v>1</v>
@@ -3764,30 +3764,30 @@
       </c>
     </row>
     <row r="12" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="162" t="s">
-        <v>62</v>
+      <c r="B12" s="152" t="s">
+        <v>56</v>
       </c>
       <c r="C12" s="116"/>
       <c r="D12" s="116"/>
       <c r="E12" s="116"/>
       <c r="F12" s="118"/>
-      <c r="G12" s="162" t="s">
-        <v>63</v>
+      <c r="G12" s="152" t="s">
+        <v>57</v>
       </c>
       <c r="H12" s="116"/>
       <c r="I12" s="116"/>
       <c r="J12" s="116"/>
       <c r="K12" s="116"/>
       <c r="L12" s="118"/>
-      <c r="M12" s="162" t="s">
-        <v>64</v>
+      <c r="M12" s="152" t="s">
+        <v>58</v>
       </c>
       <c r="N12" s="116"/>
       <c r="O12" s="116"/>
       <c r="P12" s="116"/>
       <c r="Q12" s="118"/>
-      <c r="R12" s="162" t="s">
-        <v>65</v>
+      <c r="R12" s="152" t="s">
+        <v>59</v>
       </c>
       <c r="S12" s="116"/>
       <c r="T12" s="116"/>
@@ -3796,33 +3796,33 @@
       <c r="W12" s="118"/>
     </row>
     <row r="13" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="148" t="s">
-        <v>66</v>
+      <c r="B13" s="151" t="s">
+        <v>60</v>
       </c>
       <c r="C13" s="116"/>
       <c r="D13" s="118"/>
-      <c r="E13" s="165">
+      <c r="E13" s="171">
         <f>Input_Bulanan!D11</f>
         <v>1</v>
       </c>
       <c r="F13" s="118"/>
-      <c r="G13" s="187" t="s">
-        <v>67</v>
+      <c r="G13" s="139" t="s">
+        <v>61</v>
       </c>
       <c r="H13" s="116"/>
       <c r="I13" s="118"/>
-      <c r="J13" s="167">
+      <c r="J13" s="162">
         <f>Input_Bulanan!D8</f>
         <v>100</v>
       </c>
       <c r="K13" s="116"/>
       <c r="L13" s="118"/>
-      <c r="M13" s="161" t="s">
-        <v>68</v>
+      <c r="M13" s="157" t="s">
+        <v>62</v>
       </c>
       <c r="N13" s="116"/>
       <c r="O13" s="118"/>
-      <c r="P13" s="188">
+      <c r="P13" s="161">
         <f>Input_Bulanan!D48</f>
         <v>5</v>
       </c>
@@ -3831,7 +3831,7 @@
         <f>Input_Bulanan!C74</f>
         <v>C1</v>
       </c>
-      <c r="S13" s="172" t="str">
+      <c r="S13" s="160" t="str">
         <f>Input_Bulanan!D74&amp;"  |  L="&amp;Input_Bulanan!F74&amp;", C="&amp;Input_Bulanan!G74&amp;", Skala="&amp;Input_Bulanan!H74&amp;" -&gt; "&amp;Input_Bulanan!I74</f>
         <v>Salt Supply Disruption (gangguan pasokan garam industri)  |  L=4, C=5, Skala=24 -&gt; High</v>
       </c>
@@ -3841,33 +3841,33 @@
       <c r="W13" s="116"/>
     </row>
     <row r="14" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="148" t="s">
-        <v>69</v>
+      <c r="B14" s="151" t="s">
+        <v>63</v>
       </c>
       <c r="C14" s="116"/>
       <c r="D14" s="118"/>
-      <c r="E14" s="165">
+      <c r="E14" s="171">
         <f>Input_Bulanan!D13</f>
         <v>1</v>
       </c>
       <c r="F14" s="118"/>
-      <c r="G14" s="187" t="s">
-        <v>70</v>
+      <c r="G14" s="139" t="s">
+        <v>64</v>
       </c>
       <c r="H14" s="116"/>
       <c r="I14" s="118"/>
-      <c r="J14" s="167">
+      <c r="J14" s="162">
         <f>Input_Bulanan!D9</f>
         <v>100</v>
       </c>
       <c r="K14" s="116"/>
       <c r="L14" s="118"/>
-      <c r="M14" s="161" t="s">
-        <v>71</v>
+      <c r="M14" s="157" t="s">
+        <v>65</v>
       </c>
       <c r="N14" s="116"/>
       <c r="O14" s="118"/>
-      <c r="P14" s="170">
+      <c r="P14" s="176">
         <f>Input_Bulanan!D49</f>
         <v>11</v>
       </c>
@@ -3876,7 +3876,7 @@
         <f>Input_Bulanan!C75</f>
         <v>C2</v>
       </c>
-      <c r="S14" s="172" t="str">
+      <c r="S14" s="160" t="str">
         <f>Input_Bulanan!D75&amp;"  |  L="&amp;Input_Bulanan!F75&amp;", C="&amp;Input_Bulanan!G75&amp;", Skala="&amp;Input_Bulanan!H75&amp;" -&gt; "&amp;Input_Bulanan!I75</f>
         <v>Commissioning Delay (keterlambatan commissioning)  |  L=5, C=5, Skala=25 -&gt; High</v>
       </c>
@@ -3886,33 +3886,33 @@
       <c r="W14" s="116"/>
     </row>
     <row r="15" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="148" t="s">
-        <v>72</v>
+      <c r="B15" s="151" t="s">
+        <v>66</v>
       </c>
       <c r="C15" s="116"/>
       <c r="D15" s="118"/>
-      <c r="E15" s="150">
+      <c r="E15" s="174">
         <f>Input_Bulanan!D12</f>
         <v>0</v>
       </c>
       <c r="F15" s="118"/>
-      <c r="G15" s="187" t="s">
-        <v>73</v>
+      <c r="G15" s="139" t="s">
+        <v>67</v>
       </c>
       <c r="H15" s="116"/>
       <c r="I15" s="118"/>
-      <c r="J15" s="167">
+      <c r="J15" s="162">
         <f>Input_Bulanan!D10</f>
         <v>100</v>
       </c>
       <c r="K15" s="116"/>
       <c r="L15" s="118"/>
-      <c r="M15" s="161" t="s">
-        <v>74</v>
+      <c r="M15" s="157" t="s">
+        <v>68</v>
       </c>
       <c r="N15" s="116"/>
       <c r="O15" s="118"/>
-      <c r="P15" s="189">
+      <c r="P15" s="163">
         <f>Input_Bulanan!D50</f>
         <v>18</v>
       </c>
@@ -3921,7 +3921,7 @@
         <f>Input_Bulanan!C76</f>
         <v>C3</v>
       </c>
-      <c r="S15" s="172" t="str">
+      <c r="S15" s="160" t="str">
         <f>Input_Bulanan!D76&amp;"  |  L="&amp;Input_Bulanan!F76&amp;", C="&amp;Input_Bulanan!G76&amp;", Skala="&amp;Input_Bulanan!H76&amp;" -&gt; "&amp;Input_Bulanan!I76</f>
         <v>EPC Interface Issue (isu EPC interface lintas kontraktor)  |  L=4, C=4, Skala=19 -&gt; Moderate to High</v>
       </c>
@@ -3931,30 +3931,30 @@
       <c r="W15" s="116"/>
     </row>
     <row r="16" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="148" t="s">
-        <v>75</v>
+      <c r="B16" s="151" t="s">
+        <v>69</v>
       </c>
       <c r="C16" s="116"/>
       <c r="D16" s="118"/>
-      <c r="E16" s="150">
+      <c r="E16" s="174">
         <f>Input_Bulanan!D14</f>
         <v>0</v>
       </c>
       <c r="F16" s="118"/>
-      <c r="G16" s="151" t="s">
-        <v>76</v>
+      <c r="G16" s="192" t="s">
+        <v>70</v>
       </c>
       <c r="H16" s="116"/>
       <c r="I16" s="116"/>
       <c r="J16" s="116"/>
       <c r="K16" s="116"/>
       <c r="L16" s="118"/>
-      <c r="M16" s="161" t="s">
-        <v>77</v>
+      <c r="M16" s="157" t="s">
+        <v>71</v>
       </c>
       <c r="N16" s="116"/>
       <c r="O16" s="118"/>
-      <c r="P16" s="145">
+      <c r="P16" s="191">
         <f>Input_Bulanan!D51</f>
         <v>4</v>
       </c>
@@ -3963,7 +3963,7 @@
         <f>Input_Bulanan!C77</f>
         <v>C4</v>
       </c>
-      <c r="S16" s="172" t="str">
+      <c r="S16" s="160" t="str">
         <f>Input_Bulanan!D77&amp;"  |  L="&amp;Input_Bulanan!F77&amp;", C="&amp;Input_Bulanan!G77&amp;", Skala="&amp;Input_Bulanan!H77&amp;" -&gt; "&amp;Input_Bulanan!I77</f>
         <v>Long Lead Equipment (keterlambatan peralatan utama)  |  L=3, C=3, Skala=13 -&gt; Moderate</v>
       </c>
@@ -3974,12 +3974,12 @@
     </row>
     <row r="17" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="L17" s="106"/>
-      <c r="M17" s="161" t="s">
-        <v>78</v>
+      <c r="M17" s="157" t="s">
+        <v>72</v>
       </c>
       <c r="N17" s="116"/>
       <c r="O17" s="118"/>
-      <c r="P17" s="145">
+      <c r="P17" s="191">
         <f>Input_Bulanan!D52</f>
         <v>3</v>
       </c>
@@ -3987,11 +3987,11 @@
     </row>
     <row r="18" spans="2:23" x14ac:dyDescent="0.45">
       <c r="M18" s="105" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="N18" s="103"/>
       <c r="O18" s="104"/>
-      <c r="P18" s="149">
+      <c r="P18" s="190">
         <f>Input_Bulanan!D53</f>
         <v>41</v>
       </c>
@@ -4016,21 +4016,21 @@
       <c r="Q19" s="114"/>
     </row>
     <row r="20" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="173" t="s">
-        <v>80</v>
-      </c>
-      <c r="C20" s="174"/>
-      <c r="D20" s="174"/>
-      <c r="E20" s="174"/>
-      <c r="F20" s="174"/>
-      <c r="G20" s="174"/>
-      <c r="H20" s="174"/>
-      <c r="I20" s="174"/>
-      <c r="J20" s="174"/>
-      <c r="K20" s="174"/>
-      <c r="L20" s="175"/>
-      <c r="M20" s="186" t="s">
-        <v>81</v>
+      <c r="B20" s="177" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="178"/>
+      <c r="D20" s="178"/>
+      <c r="E20" s="178"/>
+      <c r="F20" s="178"/>
+      <c r="G20" s="178"/>
+      <c r="H20" s="178"/>
+      <c r="I20" s="178"/>
+      <c r="J20" s="178"/>
+      <c r="K20" s="178"/>
+      <c r="L20" s="179"/>
+      <c r="M20" s="172" t="s">
+        <v>75</v>
       </c>
       <c r="N20" s="116"/>
       <c r="O20" s="116"/>
@@ -4038,92 +4038,92 @@
       <c r="Q20" s="118"/>
     </row>
     <row r="21" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="176"/>
-      <c r="C21" s="177"/>
-      <c r="D21" s="177"/>
-      <c r="E21" s="177"/>
-      <c r="F21" s="177"/>
-      <c r="G21" s="177"/>
-      <c r="H21" s="177"/>
-      <c r="I21" s="177"/>
-      <c r="J21" s="177"/>
-      <c r="K21" s="177"/>
-      <c r="L21" s="178"/>
-      <c r="M21" s="148" t="s">
-        <v>82</v>
+      <c r="B21" s="180"/>
+      <c r="C21" s="181"/>
+      <c r="D21" s="181"/>
+      <c r="E21" s="181"/>
+      <c r="F21" s="181"/>
+      <c r="G21" s="181"/>
+      <c r="H21" s="181"/>
+      <c r="I21" s="181"/>
+      <c r="J21" s="181"/>
+      <c r="K21" s="181"/>
+      <c r="L21" s="182"/>
+      <c r="M21" s="151" t="s">
+        <v>76</v>
       </c>
       <c r="N21" s="116"/>
       <c r="O21" s="118"/>
-      <c r="P21" s="163">
+      <c r="P21" s="149">
         <f>Input_Bulanan!D56</f>
         <v>0.82</v>
       </c>
       <c r="Q21" s="118"/>
     </row>
     <row r="22" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="176"/>
-      <c r="C22" s="177"/>
-      <c r="D22" s="177"/>
-      <c r="E22" s="177"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="177"/>
-      <c r="K22" s="177"/>
-      <c r="L22" s="178"/>
-      <c r="M22" s="148" t="s">
-        <v>83</v>
+      <c r="B22" s="180"/>
+      <c r="C22" s="181"/>
+      <c r="D22" s="181"/>
+      <c r="E22" s="181"/>
+      <c r="F22" s="181"/>
+      <c r="G22" s="181"/>
+      <c r="H22" s="181"/>
+      <c r="I22" s="181"/>
+      <c r="J22" s="181"/>
+      <c r="K22" s="181"/>
+      <c r="L22" s="182"/>
+      <c r="M22" s="151" t="s">
+        <v>77</v>
       </c>
       <c r="N22" s="116"/>
       <c r="O22" s="118"/>
-      <c r="P22" s="163">
+      <c r="P22" s="149">
         <f>Input_Bulanan!D57</f>
         <v>0.18</v>
       </c>
       <c r="Q22" s="118"/>
     </row>
     <row r="23" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="176"/>
-      <c r="C23" s="177"/>
-      <c r="D23" s="177"/>
-      <c r="E23" s="177"/>
-      <c r="F23" s="177"/>
-      <c r="G23" s="177"/>
-      <c r="H23" s="177"/>
-      <c r="I23" s="177"/>
-      <c r="J23" s="177"/>
-      <c r="K23" s="177"/>
-      <c r="L23" s="178"/>
-      <c r="M23" s="148" t="s">
-        <v>84</v>
+      <c r="B23" s="180"/>
+      <c r="C23" s="181"/>
+      <c r="D23" s="181"/>
+      <c r="E23" s="181"/>
+      <c r="F23" s="181"/>
+      <c r="G23" s="181"/>
+      <c r="H23" s="181"/>
+      <c r="I23" s="181"/>
+      <c r="J23" s="181"/>
+      <c r="K23" s="181"/>
+      <c r="L23" s="182"/>
+      <c r="M23" s="151" t="s">
+        <v>78</v>
       </c>
       <c r="N23" s="116"/>
       <c r="O23" s="118"/>
-      <c r="P23" s="163">
+      <c r="P23" s="149">
         <f>Input_Bulanan!D58</f>
         <v>0.76</v>
       </c>
       <c r="Q23" s="118"/>
     </row>
     <row r="24" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="179"/>
-      <c r="C24" s="180"/>
-      <c r="D24" s="180"/>
-      <c r="E24" s="180"/>
-      <c r="F24" s="180"/>
-      <c r="G24" s="180"/>
-      <c r="H24" s="180"/>
-      <c r="I24" s="180"/>
-      <c r="J24" s="180"/>
-      <c r="K24" s="180"/>
-      <c r="L24" s="181"/>
-      <c r="M24" s="148" t="s">
-        <v>85</v>
+      <c r="B24" s="183"/>
+      <c r="C24" s="184"/>
+      <c r="D24" s="184"/>
+      <c r="E24" s="184"/>
+      <c r="F24" s="184"/>
+      <c r="G24" s="184"/>
+      <c r="H24" s="184"/>
+      <c r="I24" s="184"/>
+      <c r="J24" s="184"/>
+      <c r="K24" s="184"/>
+      <c r="L24" s="185"/>
+      <c r="M24" s="151" t="s">
+        <v>79</v>
       </c>
       <c r="N24" s="116"/>
       <c r="O24" s="118"/>
-      <c r="P24" s="183">
+      <c r="P24" s="168">
         <f>Input_Bulanan!D59</f>
         <v>5</v>
       </c>
@@ -4154,8 +4154,8 @@
       <c r="W25" s="114"/>
     </row>
     <row r="26" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="166" t="s">
-        <v>86</v>
+      <c r="B26" s="158" t="s">
+        <v>80</v>
       </c>
       <c r="C26" s="116"/>
       <c r="D26" s="116"/>
@@ -4180,34 +4180,34 @@
       <c r="W26" s="118"/>
     </row>
     <row r="27" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="164" t="s">
-        <v>87</v>
+      <c r="B27" s="147" t="s">
+        <v>81</v>
       </c>
       <c r="C27" s="116"/>
       <c r="D27" s="116"/>
       <c r="E27" s="116"/>
       <c r="F27" s="118"/>
-      <c r="G27" s="164" t="s">
-        <v>88</v>
+      <c r="G27" s="147" t="s">
+        <v>82</v>
       </c>
       <c r="H27" s="116"/>
       <c r="I27" s="116"/>
       <c r="J27" s="118"/>
-      <c r="K27" s="164" t="s">
-        <v>89</v>
+      <c r="K27" s="147" t="s">
+        <v>83</v>
       </c>
       <c r="L27" s="118"/>
       <c r="M27" s="12" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="O27" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="P27" s="164" t="s">
-        <v>93</v>
+        <v>86</v>
+      </c>
+      <c r="P27" s="147" t="s">
+        <v>87</v>
       </c>
       <c r="Q27" s="116"/>
       <c r="R27" s="116"/>
@@ -4218,20 +4218,20 @@
       <c r="W27" s="118"/>
     </row>
     <row r="28" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="187" t="s">
-        <v>94</v>
+      <c r="B28" s="139" t="s">
+        <v>88</v>
       </c>
       <c r="C28" s="116"/>
       <c r="D28" s="116"/>
       <c r="E28" s="116"/>
       <c r="F28" s="118"/>
-      <c r="G28" s="140" t="s">
-        <v>95</v>
+      <c r="G28" s="150" t="s">
+        <v>89</v>
       </c>
       <c r="H28" s="116"/>
       <c r="I28" s="116"/>
       <c r="J28" s="118"/>
-      <c r="K28" s="184">
+      <c r="K28" s="169">
         <f>Input_Bulanan!E63</f>
         <v>24</v>
       </c>
@@ -4248,8 +4248,8 @@
         <f>IF(Input_Bulanan!H63="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P28" s="139" t="s">
-        <v>96</v>
+      <c r="P28" s="189" t="s">
+        <v>90</v>
       </c>
       <c r="Q28" s="116"/>
       <c r="R28" s="116"/>
@@ -4260,20 +4260,20 @@
       <c r="W28" s="118"/>
     </row>
     <row r="29" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="138" t="s">
-        <v>97</v>
+      <c r="B29" s="153" t="s">
+        <v>91</v>
       </c>
       <c r="C29" s="116"/>
       <c r="D29" s="116"/>
       <c r="E29" s="116"/>
       <c r="F29" s="118"/>
-      <c r="G29" s="171" t="s">
-        <v>98</v>
+      <c r="G29" s="165" t="s">
+        <v>92</v>
       </c>
       <c r="H29" s="116"/>
       <c r="I29" s="116"/>
       <c r="J29" s="118"/>
-      <c r="K29" s="146">
+      <c r="K29" s="140">
         <f>Input_Bulanan!E64</f>
         <v>0.73</v>
       </c>
@@ -4290,8 +4290,8 @@
         <f>IF(Input_Bulanan!H64="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P29" s="169" t="s">
-        <v>99</v>
+      <c r="P29" s="164" t="s">
+        <v>93</v>
       </c>
       <c r="Q29" s="116"/>
       <c r="R29" s="116"/>
@@ -4302,20 +4302,20 @@
       <c r="W29" s="118"/>
     </row>
     <row r="30" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="187" t="s">
-        <v>100</v>
+      <c r="B30" s="139" t="s">
+        <v>94</v>
       </c>
       <c r="C30" s="116"/>
       <c r="D30" s="116"/>
       <c r="E30" s="116"/>
       <c r="F30" s="118"/>
-      <c r="G30" s="140" t="s">
-        <v>101</v>
+      <c r="G30" s="150" t="s">
+        <v>95</v>
       </c>
       <c r="H30" s="116"/>
       <c r="I30" s="116"/>
       <c r="J30" s="118"/>
-      <c r="K30" s="185">
+      <c r="K30" s="170">
         <f>Input_Bulanan!E65</f>
         <v>0.94</v>
       </c>
@@ -4332,8 +4332,8 @@
         <f>IF(Input_Bulanan!H65="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P30" s="139" t="s">
-        <v>102</v>
+      <c r="P30" s="189" t="s">
+        <v>96</v>
       </c>
       <c r="Q30" s="116"/>
       <c r="R30" s="116"/>
@@ -4344,20 +4344,20 @@
       <c r="W30" s="118"/>
     </row>
     <row r="31" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="138" t="s">
-        <v>103</v>
+      <c r="B31" s="153" t="s">
+        <v>97</v>
       </c>
       <c r="C31" s="116"/>
       <c r="D31" s="116"/>
       <c r="E31" s="116"/>
       <c r="F31" s="118"/>
-      <c r="G31" s="171" t="s">
-        <v>104</v>
+      <c r="G31" s="165" t="s">
+        <v>98</v>
       </c>
       <c r="H31" s="116"/>
       <c r="I31" s="116"/>
       <c r="J31" s="118"/>
-      <c r="K31" s="146">
+      <c r="K31" s="140">
         <f>Input_Bulanan!E66</f>
         <v>0.75</v>
       </c>
@@ -4374,8 +4374,8 @@
         <f>IF(Input_Bulanan!H66="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P31" s="169" t="s">
-        <v>105</v>
+      <c r="P31" s="164" t="s">
+        <v>99</v>
       </c>
       <c r="Q31" s="116"/>
       <c r="R31" s="116"/>
@@ -4386,20 +4386,20 @@
       <c r="W31" s="118"/>
     </row>
     <row r="32" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="187" t="s">
-        <v>106</v>
+      <c r="B32" s="139" t="s">
+        <v>100</v>
       </c>
       <c r="C32" s="116"/>
       <c r="D32" s="116"/>
       <c r="E32" s="116"/>
       <c r="F32" s="118"/>
-      <c r="G32" s="140" t="s">
-        <v>107</v>
+      <c r="G32" s="150" t="s">
+        <v>101</v>
       </c>
       <c r="H32" s="116"/>
       <c r="I32" s="116"/>
       <c r="J32" s="118"/>
-      <c r="K32" s="190">
+      <c r="K32" s="166">
         <f>Input_Bulanan!E67</f>
         <v>0.42</v>
       </c>
@@ -4416,8 +4416,8 @@
         <f>IF(Input_Bulanan!H67="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P32" s="139" t="s">
-        <v>108</v>
+      <c r="P32" s="189" t="s">
+        <v>102</v>
       </c>
       <c r="Q32" s="116"/>
       <c r="R32" s="116"/>
@@ -4428,20 +4428,20 @@
       <c r="W32" s="118"/>
     </row>
     <row r="33" spans="2:23" x14ac:dyDescent="0.45">
-      <c r="B33" s="138" t="s">
-        <v>109</v>
+      <c r="B33" s="153" t="s">
+        <v>103</v>
       </c>
       <c r="C33" s="116"/>
       <c r="D33" s="116"/>
       <c r="E33" s="116"/>
       <c r="F33" s="118"/>
-      <c r="G33" s="171" t="s">
-        <v>110</v>
+      <c r="G33" s="165" t="s">
+        <v>104</v>
       </c>
       <c r="H33" s="116"/>
       <c r="I33" s="116"/>
       <c r="J33" s="118"/>
-      <c r="K33" s="146">
+      <c r="K33" s="140">
         <f>Input_Bulanan!E68</f>
         <v>0.4</v>
       </c>
@@ -4458,8 +4458,8 @@
         <f>IF(Input_Bulanan!H68="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P33" s="169" t="s">
-        <v>111</v>
+      <c r="P33" s="164" t="s">
+        <v>105</v>
       </c>
       <c r="Q33" s="116"/>
       <c r="R33" s="116"/>
@@ -4494,8 +4494,8 @@
       <c r="W34" s="114"/>
     </row>
     <row r="35" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="166" t="s">
-        <v>112</v>
+      <c r="B35" s="158" t="s">
+        <v>106</v>
       </c>
       <c r="C35" s="116"/>
       <c r="D35" s="116"/>
@@ -4520,7 +4520,7 @@
       <c r="W35" s="118"/>
     </row>
     <row r="36" spans="2:23" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="154" t="str">
+      <c r="B36" s="159" t="str">
         <f>"Prioritas 1—2: [1] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 1), Risk_Action_Tracker!Z$6:Z$15, 0)) &amp; " · [2] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 2), Risk_Action_Tracker!Z$6:Z$15, 0))</f>
         <v>Prioritas 1—2: [1] Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A. · [2] Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Perusahaan Induk X (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</v>
       </c>
@@ -4547,8 +4547,8 @@
       <c r="W36" s="118"/>
     </row>
     <row r="37" spans="2:23" ht="42.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="154" t="s">
-        <v>113</v>
+      <c r="B37" s="159" t="s">
+        <v>107</v>
       </c>
       <c r="C37" s="116"/>
       <c r="D37" s="116"/>
@@ -4574,6 +4574,88 @@
     </row>
   </sheetData>
   <mergeCells count="98">
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="P30:W30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="K6:L7"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P32:W32"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="P28:W28"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="B2:W2"/>
+    <mergeCell ref="B34:W34"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B37:W37"/>
+    <mergeCell ref="M6:Q9"/>
+    <mergeCell ref="G8:J9"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="G10:J11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="P21:Q21"/>
+    <mergeCell ref="P27:W27"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="B35:W35"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="B25:W25"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="M10:Q11"/>
+    <mergeCell ref="P33:W33"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="S16:W16"/>
+    <mergeCell ref="B20:L24"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="P29:W29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B36:W36"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="K10:L11"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="S15:W15"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P31:W31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K32:L32"/>
     <mergeCell ref="M4:W4"/>
     <mergeCell ref="G13:I13"/>
     <mergeCell ref="K33:L33"/>
@@ -4590,88 +4672,6 @@
     <mergeCell ref="B6:F9"/>
     <mergeCell ref="M17:O17"/>
     <mergeCell ref="B26:W26"/>
-    <mergeCell ref="B36:W36"/>
-    <mergeCell ref="S14:W14"/>
-    <mergeCell ref="K10:L11"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="S15:W15"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="P31:W31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="P29:W29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="R12:W12"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B35:W35"/>
-    <mergeCell ref="G6:J7"/>
-    <mergeCell ref="B25:W25"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="M10:Q11"/>
-    <mergeCell ref="P33:W33"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="S16:W16"/>
-    <mergeCell ref="B20:L24"/>
-    <mergeCell ref="B2:W2"/>
-    <mergeCell ref="B34:W34"/>
-    <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B37:W37"/>
-    <mergeCell ref="M6:Q9"/>
-    <mergeCell ref="G8:J9"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="G10:J11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="P21:Q21"/>
-    <mergeCell ref="P27:W27"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="P28:W28"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B19:L19"/>
-    <mergeCell ref="G16:L16"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="P30:W30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="K6:L7"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P32:W32"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:F11">
     <cfRule type="expression" dxfId="11" priority="2">
@@ -4742,7 +4742,7 @@
   <sheetData>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="13" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -4750,8 +4750,8 @@
       <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="125" t="s">
-        <v>390</v>
+      <c r="A3" s="133" t="s">
+        <v>384</v>
       </c>
       <c r="B3" s="114"/>
       <c r="C3" s="114"/>
@@ -4759,8 +4759,8 @@
       <c r="E3" s="114"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="120" t="s">
-        <v>115</v>
+      <c r="A5" s="117" t="s">
+        <v>109</v>
       </c>
       <c r="B5" s="116"/>
       <c r="C5" s="116"/>
@@ -4769,53 +4769,53 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="14" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="19" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D8" s="110">
         <v>0.2</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4823,50 +4823,50 @@
         <v>53</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D9" s="110">
         <v>0.2</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D10" s="110">
         <v>0.2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D11" s="110">
         <v>0.2</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4878,8 +4878,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="113" t="s">
-        <v>136</v>
+      <c r="A14" s="137" t="s">
+        <v>130</v>
       </c>
       <c r="B14" s="114"/>
       <c r="C14" s="114"/>
@@ -4887,8 +4887,8 @@
       <c r="E14" s="114"/>
     </row>
     <row r="15" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="134" t="s">
-        <v>137</v>
+      <c r="A15" s="113" t="s">
+        <v>131</v>
       </c>
       <c r="B15" s="114"/>
       <c r="C15" s="114"/>
@@ -4896,8 +4896,8 @@
       <c r="E15" s="114"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="120" t="s">
-        <v>138</v>
+      <c r="A17" s="117" t="s">
+        <v>132</v>
       </c>
       <c r="B17" s="116"/>
       <c r="C17" s="116"/>
@@ -4906,85 +4906,85 @@
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="14" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="C18" s="122" t="s">
-        <v>140</v>
+        <v>133</v>
+      </c>
+      <c r="C18" s="135" t="s">
+        <v>134</v>
       </c>
       <c r="D18" s="116"/>
       <c r="E18" s="118"/>
     </row>
     <row r="19" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="15" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B19" s="110">
         <v>0.25</v>
       </c>
-      <c r="C19" s="123" t="s">
-        <v>142</v>
+      <c r="C19" s="122" t="s">
+        <v>136</v>
       </c>
       <c r="D19" s="116"/>
       <c r="E19" s="116"/>
     </row>
     <row r="20" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="19" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B20" s="111">
         <v>0.2</v>
       </c>
       <c r="C20" s="115" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D20" s="116"/>
       <c r="E20" s="116"/>
     </row>
     <row r="21" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="15" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B21" s="110">
         <v>0.2</v>
       </c>
-      <c r="C21" s="123" t="s">
-        <v>146</v>
+      <c r="C21" s="122" t="s">
+        <v>140</v>
       </c>
       <c r="D21" s="116"/>
       <c r="E21" s="116"/>
     </row>
     <row r="22" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="19" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B22" s="111">
         <v>0.2</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D22" s="116"/>
       <c r="E22" s="116"/>
     </row>
     <row r="23" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B23" s="110">
         <v>0.15</v>
       </c>
-      <c r="C23" s="123" t="s">
-        <v>150</v>
+      <c r="C23" s="122" t="s">
+        <v>144</v>
       </c>
       <c r="D23" s="116"/>
       <c r="E23" s="116"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="120" t="s">
-        <v>151</v>
+      <c r="A25" s="117" t="s">
+        <v>145</v>
       </c>
       <c r="B25" s="116"/>
       <c r="C25" s="116"/>
@@ -4993,72 +4993,72 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="14" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="C26" s="122" t="s">
-        <v>140</v>
+        <v>133</v>
+      </c>
+      <c r="C26" s="135" t="s">
+        <v>134</v>
       </c>
       <c r="D26" s="116"/>
       <c r="E26" s="118"/>
     </row>
     <row r="27" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="15" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B27" s="110">
         <v>0.25</v>
       </c>
-      <c r="C27" s="123" t="s">
-        <v>153</v>
+      <c r="C27" s="122" t="s">
+        <v>147</v>
       </c>
       <c r="D27" s="116"/>
       <c r="E27" s="116"/>
     </row>
     <row r="28" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="19" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B28" s="111">
         <v>0.3</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D28" s="116"/>
       <c r="E28" s="116"/>
     </row>
     <row r="29" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="15" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B29" s="110">
         <v>0.35</v>
       </c>
-      <c r="C29" s="123" t="s">
-        <v>157</v>
+      <c r="C29" s="122" t="s">
+        <v>151</v>
       </c>
       <c r="D29" s="116"/>
       <c r="E29" s="116"/>
     </row>
     <row r="30" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="19" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B30" s="111">
         <v>0.1</v>
       </c>
       <c r="C30" s="115" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D30" s="116"/>
       <c r="E30" s="116"/>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="120" t="s">
-        <v>160</v>
+      <c r="A32" s="117" t="s">
+        <v>154</v>
       </c>
       <c r="B32" s="116"/>
       <c r="C32" s="116"/>
@@ -5067,85 +5067,85 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="14" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="C33" s="122" t="s">
-        <v>140</v>
+        <v>133</v>
+      </c>
+      <c r="C33" s="135" t="s">
+        <v>134</v>
       </c>
       <c r="D33" s="116"/>
       <c r="E33" s="118"/>
     </row>
     <row r="34" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="19" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B34" s="111">
         <v>0.2</v>
       </c>
       <c r="C34" s="115" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D34" s="116"/>
       <c r="E34" s="116"/>
     </row>
     <row r="35" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="15" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B35" s="110">
         <v>0.2</v>
       </c>
-      <c r="C35" s="123" t="s">
-        <v>164</v>
+      <c r="C35" s="122" t="s">
+        <v>158</v>
       </c>
       <c r="D35" s="116"/>
       <c r="E35" s="116"/>
     </row>
     <row r="36" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="19" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B36" s="111">
         <v>0.15</v>
       </c>
       <c r="C36" s="115" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D36" s="116"/>
       <c r="E36" s="116"/>
     </row>
     <row r="37" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="15" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B37" s="110">
         <v>0.2</v>
       </c>
-      <c r="C37" s="123" t="s">
-        <v>168</v>
+      <c r="C37" s="122" t="s">
+        <v>162</v>
       </c>
       <c r="D37" s="116"/>
       <c r="E37" s="116"/>
     </row>
     <row r="38" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="19" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B38" s="111">
         <v>0.25</v>
       </c>
       <c r="C38" s="115" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D38" s="116"/>
       <c r="E38" s="116"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="120" t="s">
-        <v>171</v>
+      <c r="A40" s="117" t="s">
+        <v>165</v>
       </c>
       <c r="B40" s="116"/>
       <c r="C40" s="116"/>
@@ -5154,147 +5154,147 @@
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="9" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="23" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C42" s="24" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="E42" s="26" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F42" s="27" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="28" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B43" s="28" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C43" s="24" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="E43" s="26" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="23" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C44" s="24" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E44" s="26" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F44" s="27" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="28" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B45" s="28" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C45" s="24" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E45" s="26" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="F45" s="27" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="23" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E46" s="26" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="28" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B47" s="28" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C47" s="24" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E47" s="26" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="F47" s="27" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="120" t="s">
-        <v>208</v>
+      <c r="A49" s="117" t="s">
+        <v>202</v>
       </c>
       <c r="B49" s="116"/>
       <c r="C49" s="116"/>
@@ -5302,8 +5302,8 @@
       <c r="E49" s="118"/>
     </row>
     <row r="50" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="129" t="s">
-        <v>391</v>
+      <c r="A50" s="134" t="s">
+        <v>385</v>
       </c>
       <c r="B50" s="114"/>
       <c r="C50" s="114"/>
@@ -5312,13 +5312,13 @@
     </row>
     <row r="51" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="9" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="117" t="s">
-        <v>210</v>
+      <c r="C51" s="121" t="s">
+        <v>204</v>
       </c>
       <c r="D51" s="116"/>
       <c r="E51" s="118"/>
@@ -5328,10 +5328,10 @@
         <v>1</v>
       </c>
       <c r="B52" s="30" t="s">
-        <v>211</v>
-      </c>
-      <c r="C52" s="121" t="s">
-        <v>212</v>
+        <v>205</v>
+      </c>
+      <c r="C52" s="120" t="s">
+        <v>206</v>
       </c>
       <c r="D52" s="116"/>
       <c r="E52" s="116"/>
@@ -5341,10 +5341,10 @@
         <v>2</v>
       </c>
       <c r="B53" s="32" t="s">
-        <v>213</v>
-      </c>
-      <c r="C53" s="119" t="s">
-        <v>214</v>
+        <v>207</v>
+      </c>
+      <c r="C53" s="127" t="s">
+        <v>208</v>
       </c>
       <c r="D53" s="116"/>
       <c r="E53" s="116"/>
@@ -5354,10 +5354,10 @@
         <v>3</v>
       </c>
       <c r="B54" s="30" t="s">
-        <v>215</v>
-      </c>
-      <c r="C54" s="121" t="s">
-        <v>216</v>
+        <v>209</v>
+      </c>
+      <c r="C54" s="120" t="s">
+        <v>210</v>
       </c>
       <c r="D54" s="116"/>
       <c r="E54" s="116"/>
@@ -5367,10 +5367,10 @@
         <v>4</v>
       </c>
       <c r="B55" s="32" t="s">
-        <v>217</v>
-      </c>
-      <c r="C55" s="119" t="s">
-        <v>218</v>
+        <v>211</v>
+      </c>
+      <c r="C55" s="127" t="s">
+        <v>212</v>
       </c>
       <c r="D55" s="116"/>
       <c r="E55" s="116"/>
@@ -5380,17 +5380,17 @@
         <v>5</v>
       </c>
       <c r="B56" s="30" t="s">
-        <v>219</v>
-      </c>
-      <c r="C56" s="121" t="s">
-        <v>220</v>
+        <v>213</v>
+      </c>
+      <c r="C56" s="120" t="s">
+        <v>214</v>
       </c>
       <c r="D56" s="116"/>
       <c r="E56" s="116"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="120" t="s">
-        <v>221</v>
+      <c r="A58" s="117" t="s">
+        <v>215</v>
       </c>
       <c r="B58" s="116"/>
       <c r="C58" s="116"/>
@@ -5399,13 +5399,13 @@
     </row>
     <row r="59" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="117" t="s">
-        <v>223</v>
+      <c r="C59" s="121" t="s">
+        <v>217</v>
       </c>
       <c r="D59" s="116"/>
       <c r="E59" s="118"/>
@@ -5415,10 +5415,10 @@
         <v>1</v>
       </c>
       <c r="B60" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="C60" s="121" t="s">
-        <v>225</v>
+        <v>218</v>
+      </c>
+      <c r="C60" s="120" t="s">
+        <v>219</v>
       </c>
       <c r="D60" s="116"/>
       <c r="E60" s="116"/>
@@ -5428,10 +5428,10 @@
         <v>2</v>
       </c>
       <c r="B61" s="32" t="s">
-        <v>226</v>
-      </c>
-      <c r="C61" s="119" t="s">
-        <v>227</v>
+        <v>220</v>
+      </c>
+      <c r="C61" s="127" t="s">
+        <v>221</v>
       </c>
       <c r="D61" s="116"/>
       <c r="E61" s="116"/>
@@ -5441,10 +5441,10 @@
         <v>3</v>
       </c>
       <c r="B62" s="30" t="s">
-        <v>228</v>
-      </c>
-      <c r="C62" s="121" t="s">
-        <v>229</v>
+        <v>222</v>
+      </c>
+      <c r="C62" s="120" t="s">
+        <v>223</v>
       </c>
       <c r="D62" s="116"/>
       <c r="E62" s="116"/>
@@ -5454,10 +5454,10 @@
         <v>4</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>230</v>
-      </c>
-      <c r="C63" s="119" t="s">
-        <v>231</v>
+        <v>224</v>
+      </c>
+      <c r="C63" s="127" t="s">
+        <v>225</v>
       </c>
       <c r="D63" s="116"/>
       <c r="E63" s="116"/>
@@ -5467,17 +5467,17 @@
         <v>5</v>
       </c>
       <c r="B64" s="30" t="s">
-        <v>232</v>
-      </c>
-      <c r="C64" s="121" t="s">
-        <v>233</v>
+        <v>226</v>
+      </c>
+      <c r="C64" s="120" t="s">
+        <v>227</v>
       </c>
       <c r="D64" s="116"/>
       <c r="E64" s="116"/>
     </row>
     <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="120" t="s">
-        <v>392</v>
+      <c r="A66" s="117" t="s">
+        <v>386</v>
       </c>
       <c r="B66" s="116"/>
       <c r="C66" s="116"/>
@@ -5485,8 +5485,8 @@
       <c r="E66" s="118"/>
     </row>
     <row r="67" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" s="130" t="s">
-        <v>234</v>
+      <c r="A67" s="136" t="s">
+        <v>228</v>
       </c>
       <c r="B67" s="114"/>
       <c r="C67" s="114"/>
@@ -5495,85 +5495,85 @@
     </row>
     <row r="68" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="9" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="C68" s="117" t="s">
-        <v>237</v>
+        <v>230</v>
+      </c>
+      <c r="C68" s="121" t="s">
+        <v>231</v>
       </c>
       <c r="D68" s="116"/>
       <c r="E68" s="118"/>
     </row>
     <row r="69" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="36" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B69" s="37" t="s">
-        <v>238</v>
-      </c>
-      <c r="C69" s="124" t="s">
-        <v>239</v>
+        <v>232</v>
+      </c>
+      <c r="C69" s="125" t="s">
+        <v>233</v>
       </c>
       <c r="D69" s="116"/>
       <c r="E69" s="116"/>
     </row>
     <row r="70" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="38" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B70" s="37" t="s">
-        <v>240</v>
-      </c>
-      <c r="C70" s="124" t="s">
-        <v>241</v>
+        <v>234</v>
+      </c>
+      <c r="C70" s="125" t="s">
+        <v>235</v>
       </c>
       <c r="D70" s="116"/>
       <c r="E70" s="116"/>
     </row>
     <row r="71" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="39" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B71" s="37" t="s">
-        <v>242</v>
-      </c>
-      <c r="C71" s="124" t="s">
-        <v>243</v>
+        <v>236</v>
+      </c>
+      <c r="C71" s="125" t="s">
+        <v>237</v>
       </c>
       <c r="D71" s="116"/>
       <c r="E71" s="116"/>
     </row>
     <row r="72" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="40" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>244</v>
-      </c>
-      <c r="C72" s="124" t="s">
-        <v>245</v>
+        <v>238</v>
+      </c>
+      <c r="C72" s="125" t="s">
+        <v>239</v>
       </c>
       <c r="D72" s="116"/>
       <c r="E72" s="116"/>
     </row>
     <row r="73" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="41" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B73" s="37" t="s">
-        <v>246</v>
-      </c>
-      <c r="C73" s="124" t="s">
-        <v>247</v>
+        <v>240</v>
+      </c>
+      <c r="C73" s="125" t="s">
+        <v>241</v>
       </c>
       <c r="D73" s="116"/>
       <c r="E73" s="116"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="120" t="s">
-        <v>248</v>
+      <c r="A75" s="117" t="s">
+        <v>242</v>
       </c>
       <c r="B75" s="116"/>
       <c r="C75" s="116"/>
@@ -5582,46 +5582,46 @@
     </row>
     <row r="76" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="19" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B76" s="111">
         <v>0.4</v>
       </c>
-      <c r="C76" s="121" t="s">
-        <v>250</v>
+      <c r="C76" s="120" t="s">
+        <v>244</v>
       </c>
       <c r="D76" s="116"/>
       <c r="E76" s="116"/>
     </row>
     <row r="77" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="15" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B77" s="110">
         <v>0.4</v>
       </c>
-      <c r="C77" s="119" t="s">
-        <v>252</v>
+      <c r="C77" s="127" t="s">
+        <v>246</v>
       </c>
       <c r="D77" s="116"/>
       <c r="E77" s="116"/>
     </row>
     <row r="78" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="19" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B78" s="111">
         <v>0.2</v>
       </c>
-      <c r="C78" s="121" t="s">
-        <v>388</v>
+      <c r="C78" s="120" t="s">
+        <v>382</v>
       </c>
       <c r="D78" s="116"/>
       <c r="E78" s="116"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="136" t="s">
-        <v>254</v>
+      <c r="A79" s="123" t="s">
+        <v>248</v>
       </c>
       <c r="B79" s="114"/>
       <c r="C79" s="114"/>
@@ -5630,7 +5630,7 @@
     </row>
     <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="42" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -5638,7 +5638,7 @@
     <row r="84" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="86" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="43" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B86" s="44"/>
       <c r="C86" s="44"/>
@@ -5647,8 +5647,8 @@
       <c r="F86" s="44"/>
     </row>
     <row r="87" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="131" t="s">
-        <v>394</v>
+      <c r="A87" s="126" t="s">
+        <v>388</v>
       </c>
       <c r="B87" s="114"/>
       <c r="C87" s="114"/>
@@ -5658,22 +5658,22 @@
     </row>
     <row r="89" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="12" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="D89" s="12" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="F89" s="12" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5690,10 +5690,10 @@
         <v>1</v>
       </c>
       <c r="E90" s="46" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F90" s="45" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5710,10 +5710,10 @@
         <v>2</v>
       </c>
       <c r="E91" s="46" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F91" s="45" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5730,10 +5730,10 @@
         <v>3</v>
       </c>
       <c r="E92" s="46" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F92" s="45" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5750,10 +5750,10 @@
         <v>4</v>
       </c>
       <c r="E93" s="46" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F93" s="45" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5770,10 +5770,10 @@
         <v>5</v>
       </c>
       <c r="E94" s="46" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F94" s="45" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5790,10 +5790,10 @@
         <v>6</v>
       </c>
       <c r="E95" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F95" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5810,10 +5810,10 @@
         <v>7</v>
       </c>
       <c r="E96" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F96" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5830,10 +5830,10 @@
         <v>8</v>
       </c>
       <c r="E97" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F97" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5850,10 +5850,10 @@
         <v>9</v>
       </c>
       <c r="E98" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5870,10 +5870,10 @@
         <v>10</v>
       </c>
       <c r="E99" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F99" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5890,10 +5890,10 @@
         <v>11</v>
       </c>
       <c r="E100" s="47" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F100" s="45" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5910,10 +5910,10 @@
         <v>12</v>
       </c>
       <c r="E101" s="48" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F101" s="45" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5930,10 +5930,10 @@
         <v>13</v>
       </c>
       <c r="E102" s="48" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F102" s="45" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5950,10 +5950,10 @@
         <v>14</v>
       </c>
       <c r="E103" s="48" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F103" s="45" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5970,10 +5970,10 @@
         <v>15</v>
       </c>
       <c r="E104" s="48" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F104" s="45" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5990,10 +5990,10 @@
         <v>16</v>
       </c>
       <c r="E105" s="49" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F105" s="45" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6010,10 +6010,10 @@
         <v>17</v>
       </c>
       <c r="E106" s="49" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6030,10 +6030,10 @@
         <v>18</v>
       </c>
       <c r="E107" s="49" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F107" s="45" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6050,10 +6050,10 @@
         <v>19</v>
       </c>
       <c r="E108" s="49" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F108" s="45" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6070,10 +6070,10 @@
         <v>20</v>
       </c>
       <c r="E109" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F109" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6090,10 +6090,10 @@
         <v>21</v>
       </c>
       <c r="E110" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F110" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6110,10 +6110,10 @@
         <v>22</v>
       </c>
       <c r="E111" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F111" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6130,10 +6130,10 @@
         <v>23</v>
       </c>
       <c r="E112" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F112" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6150,10 +6150,10 @@
         <v>24</v>
       </c>
       <c r="E113" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F113" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -6170,15 +6170,15 @@
         <v>25</v>
       </c>
       <c r="E114" s="50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F114" s="45" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="116" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" s="131" t="s">
-        <v>395</v>
+      <c r="A116" s="126" t="s">
+        <v>389</v>
       </c>
       <c r="B116" s="114"/>
       <c r="C116" s="114"/>
@@ -6188,7 +6188,7 @@
     </row>
     <row r="118" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="43" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B118" s="44"/>
       <c r="C118" s="44"/>
@@ -6197,8 +6197,8 @@
       <c r="F118" s="44"/>
     </row>
     <row r="119" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" s="131" t="s">
-        <v>267</v>
+      <c r="A119" s="126" t="s">
+        <v>261</v>
       </c>
       <c r="B119" s="114"/>
       <c r="C119" s="114"/>
@@ -6208,53 +6208,53 @@
     </row>
     <row r="121" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="51" t="s">
-        <v>268</v>
-      </c>
-      <c r="B121" s="133" t="s">
-        <v>269</v>
+        <v>262</v>
+      </c>
+      <c r="B121" s="129" t="s">
+        <v>263</v>
       </c>
       <c r="C121" s="114"/>
       <c r="D121" s="114"/>
       <c r="E121" s="51" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="52" t="s">
-        <v>90</v>
-      </c>
-      <c r="B122" s="126" t="s">
-        <v>271</v>
-      </c>
-      <c r="C122" s="127"/>
-      <c r="D122" s="128"/>
+        <v>84</v>
+      </c>
+      <c r="B122" s="130" t="s">
+        <v>265</v>
+      </c>
+      <c r="C122" s="131"/>
+      <c r="D122" s="132"/>
       <c r="E122" s="53"/>
     </row>
     <row r="123" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="54" t="s">
-        <v>91</v>
-      </c>
-      <c r="B123" s="126" t="s">
-        <v>272</v>
-      </c>
-      <c r="C123" s="127"/>
-      <c r="D123" s="128"/>
+        <v>85</v>
+      </c>
+      <c r="B123" s="130" t="s">
+        <v>266</v>
+      </c>
+      <c r="C123" s="131"/>
+      <c r="D123" s="132"/>
       <c r="E123" s="53"/>
     </row>
     <row r="124" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="55" t="s">
-        <v>92</v>
-      </c>
-      <c r="B124" s="126" t="s">
-        <v>273</v>
-      </c>
-      <c r="C124" s="127"/>
-      <c r="D124" s="128"/>
+        <v>86</v>
+      </c>
+      <c r="B124" s="130" t="s">
+        <v>267</v>
+      </c>
+      <c r="C124" s="131"/>
+      <c r="D124" s="132"/>
       <c r="E124" s="53"/>
     </row>
     <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A127" s="93" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B127" s="94"/>
       <c r="C127" s="94"/>
@@ -6263,8 +6263,8 @@
       <c r="F127" s="94"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A129" s="137" t="s">
-        <v>275</v>
+      <c r="A129" s="124" t="s">
+        <v>269</v>
       </c>
       <c r="B129" s="114"/>
       <c r="C129" s="114"/>
@@ -6274,87 +6274,87 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A130" s="95" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="B130" s="95" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C130" s="95" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="D130" s="95" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="E130" s="95" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="F130" s="95" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="96" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B131" s="96" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C131" s="96" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="D131" s="96" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="E131" s="96" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="F131" s="96" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="96" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B132" s="96" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C132" s="96" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="D132" s="96" t="s">
+        <v>278</v>
+      </c>
+      <c r="E132" s="96" t="s">
+        <v>283</v>
+      </c>
+      <c r="F132" s="96" t="s">
         <v>284</v>
-      </c>
-      <c r="E132" s="96" t="s">
-        <v>289</v>
-      </c>
-      <c r="F132" s="96" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="96" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B133" s="96" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="C133" s="96" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D133" s="96" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="E133" s="96" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="F133" s="96" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A136" s="135" t="s">
-        <v>294</v>
+      <c r="A136" s="119" t="s">
+        <v>288</v>
       </c>
       <c r="B136" s="114"/>
       <c r="C136" s="114"/>
@@ -6364,7 +6364,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A139" s="93" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="B139" s="94"/>
       <c r="C139" s="94"/>
@@ -6373,8 +6373,8 @@
       <c r="F139" s="94"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A141" s="132" t="s">
-        <v>397</v>
+      <c r="A141" s="128" t="s">
+        <v>391</v>
       </c>
       <c r="B141" s="114"/>
       <c r="C141" s="114"/>
@@ -6384,72 +6384,119 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A143" s="95" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B143" s="95" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C143" s="95" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A144" s="97" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B144" s="98" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="C144" s="98" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A145" s="99" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B145" s="98" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C145" s="98" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A146" s="100" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B146" s="98" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C146" s="98" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="101" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B147" s="98" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C147" s="98" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A148" s="102" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B148" s="98" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C148" s="98" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B123:D123"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="B122:D122"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="C63:E63"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="A49:E49"/>
@@ -6466,53 +6513,6 @@
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="C76:E76"/>
     <mergeCell ref="C71:E71"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="A141:F141"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="B121:D121"/>
-    <mergeCell ref="B122:D122"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A87:F87"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B123:D123"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C64:E64"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6543,12 +6543,12 @@
   <sheetData>
     <row r="2" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="C2" s="13" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="125" t="s">
-        <v>308</v>
+      <c r="C3" s="133" t="s">
+        <v>302</v>
       </c>
       <c r="D3" s="114"/>
       <c r="E3" s="114"/>
@@ -6557,21 +6557,21 @@
     </row>
     <row r="5" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C5" s="56" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="D5" s="57" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="E5" s="56" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="F5" s="57" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C7" s="193" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="D7" s="114"/>
       <c r="E7" s="114"/>
@@ -6580,18 +6580,18 @@
     </row>
     <row r="8" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C8" s="58" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="D8" s="59">
         <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="9" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C9" s="58" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="D9" s="59">
         <v>100</v>
@@ -6599,7 +6599,7 @@
     </row>
     <row r="10" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C10" s="58" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="D10" s="59">
         <v>100</v>
@@ -6607,7 +6607,7 @@
     </row>
     <row r="11" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C11" s="56" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D11" s="60">
         <f>D9/D10</f>
@@ -6616,7 +6616,7 @@
     </row>
     <row r="12" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C12" s="56" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="D12" s="61">
         <f>D9-D10</f>
@@ -6625,7 +6625,7 @@
     </row>
     <row r="13" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C13" s="56" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D13" s="60">
         <f>D9/D8</f>
@@ -6634,7 +6634,7 @@
     </row>
     <row r="14" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C14" s="56" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="D14" s="61">
         <f>D9-D8</f>
@@ -6643,7 +6643,7 @@
     </row>
     <row r="16" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C16" s="193" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="D16" s="114"/>
       <c r="E16" s="114"/>
@@ -6652,7 +6652,7 @@
     </row>
     <row r="17" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C17" s="58" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="D17" s="62">
         <v>0.1</v>
@@ -6660,18 +6660,18 @@
     </row>
     <row r="18" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C18" s="58" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="D18" s="62">
         <v>0.05</v>
       </c>
       <c r="E18" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
     </row>
     <row r="19" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C19" s="58" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="D19" s="62">
         <v>0.04</v>
@@ -6679,7 +6679,7 @@
     </row>
     <row r="20" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C20" s="58" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="D20" s="62">
         <v>0.06</v>
@@ -6687,7 +6687,7 @@
     </row>
     <row r="21" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C21" s="58" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="D21" s="62">
         <v>0.08</v>
@@ -6695,7 +6695,7 @@
     </row>
     <row r="22" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C22" s="56" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="D22" s="63">
         <f>(D17*0.25+D18*0.2+D19*0.2+D20*0.2+D21*0.15)</f>
@@ -6704,7 +6704,7 @@
     </row>
     <row r="24" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C24" s="193" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="D24" s="114"/>
       <c r="E24" s="114"/>
@@ -6713,82 +6713,82 @@
     </row>
     <row r="25" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C25" s="58" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="D25" s="62">
         <v>0.88</v>
       </c>
       <c r="F25" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C26" s="58" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="D26" s="62">
         <v>0.73</v>
       </c>
       <c r="F26" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="27" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C27" s="58" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="D27" s="62">
         <v>0.82</v>
       </c>
       <c r="F27" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C28" s="58" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="D28" s="62">
         <v>0.42</v>
       </c>
       <c r="E28" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="F28" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
     </row>
     <row r="29" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C29" s="56" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="D29" s="63">
         <f>(D25*0.25+D26*0.3+D27*0.35+D28*0.1)</f>
         <v>0.76800000000000002</v>
       </c>
       <c r="F29" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
     </row>
     <row r="30" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C30" s="58" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="D30" s="62">
         <v>5.8000000000000003E-2</v>
       </c>
       <c r="F30" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
     </row>
     <row r="31" spans="3:7" x14ac:dyDescent="0.45">
       <c r="F31" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="32" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C32" s="193" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="D32" s="114"/>
       <c r="E32" s="114"/>
@@ -6797,7 +6797,7 @@
     </row>
     <row r="33" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C33" s="58" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="D33" s="62">
         <v>0.6</v>
@@ -6805,7 +6805,7 @@
     </row>
     <row r="34" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C34" s="58" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="D34" s="62">
         <v>0.6</v>
@@ -6813,7 +6813,7 @@
     </row>
     <row r="35" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C35" s="58" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="D35" s="62">
         <v>0.8</v>
@@ -6821,7 +6821,7 @@
     </row>
     <row r="36" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C36" s="58" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="D36" s="62">
         <v>0.8</v>
@@ -6829,21 +6829,21 @@
     </row>
     <row r="37" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C37" s="58" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="D37" s="62">
         <v>0.4</v>
       </c>
       <c r="E37" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="F37" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
     </row>
     <row r="38" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C38" s="56" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="D38" s="63">
         <f>(D33*0.2+D34*0.2+D35*0.15+D36*0.2+D37*0.25)</f>
@@ -6852,7 +6852,7 @@
     </row>
     <row r="40" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C40" s="193" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="D40" s="114"/>
       <c r="E40" s="114"/>
@@ -6861,7 +6861,7 @@
     </row>
     <row r="41" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C41" s="58" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="D41" s="108">
         <f>D22*100</f>
@@ -6870,7 +6870,7 @@
     </row>
     <row r="42" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C42" s="58" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="D42" s="108">
         <f>D29*100</f>
@@ -6879,7 +6879,7 @@
     </row>
     <row r="43" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C43" s="58" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="D43" s="108">
         <f>D38*100</f>
@@ -6888,7 +6888,7 @@
     </row>
     <row r="44" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C44" s="56" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="D44" s="109">
         <f>(D41*0.4)+(D42*0.4)+(D43*0.2)</f>
@@ -6897,7 +6897,7 @@
     </row>
     <row r="45" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C45" s="56" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="D45" s="65" t="str">
         <f>IF(D44&lt;=20,"Low",IF(D44&lt;=44,"Low to Moderate",IF(D44&lt;=60,"Moderate",IF(D44&lt;=76,"Moderate to High","High"))))</f>
@@ -6906,7 +6906,7 @@
     </row>
     <row r="47" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C47" s="193" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="D47" s="114"/>
       <c r="E47" s="114"/>
@@ -6915,7 +6915,7 @@
     </row>
     <row r="48" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C48" s="87" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D48" s="66">
         <v>5</v>
@@ -6923,7 +6923,7 @@
     </row>
     <row r="49" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C49" s="88" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D49" s="66">
         <v>11</v>
@@ -6931,7 +6931,7 @@
     </row>
     <row r="50" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C50" s="89" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D50" s="66">
         <v>18</v>
@@ -6939,7 +6939,7 @@
     </row>
     <row r="51" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C51" s="90" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D51" s="66">
         <v>4</v>
@@ -6947,7 +6947,7 @@
     </row>
     <row r="52" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C52" s="86" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D52" s="66">
         <v>3</v>
@@ -6955,7 +6955,7 @@
     </row>
     <row r="53" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C53" s="91" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D53" s="92">
         <f>SUM(D48:D52)</f>
@@ -6971,7 +6971,7 @@
     </row>
     <row r="55" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C55" s="193" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="D55" s="114"/>
       <c r="E55" s="114"/>
@@ -6980,7 +6980,7 @@
     </row>
     <row r="56" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C56" s="58" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="D56" s="62">
         <v>0.82</v>
@@ -6994,7 +6994,7 @@
     </row>
     <row r="57" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C57" s="58" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="D57" s="62">
         <v>0.18</v>
@@ -7008,7 +7008,7 @@
     </row>
     <row r="58" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C58" s="58" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="D58" s="62">
         <v>0.76</v>
@@ -7022,7 +7022,7 @@
     </row>
     <row r="59" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C59" s="58" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D59" s="66">
         <v>5</v>
@@ -7043,7 +7043,7 @@
     </row>
     <row r="61" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C61" s="193" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="D61" s="114"/>
       <c r="E61" s="114"/>
@@ -7052,30 +7052,30 @@
     </row>
     <row r="62" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C62" s="14" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="F62" s="67" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="G62" s="67" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="H62" s="67" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="63" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C63" s="58" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D63" s="68" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="E63" s="66">
         <v>24</v>
@@ -7094,10 +7094,10 @@
     </row>
     <row r="64" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C64" s="58" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D64" s="68" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="E64" s="62">
         <v>0.73</v>
@@ -7116,10 +7116,10 @@
     </row>
     <row r="65" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C65" s="58" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D65" s="68" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E65" s="64">
         <v>0.94</v>
@@ -7138,10 +7138,10 @@
     </row>
     <row r="66" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C66" s="58" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D66" s="68" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E66" s="62">
         <v>0.75</v>
@@ -7160,10 +7160,10 @@
     </row>
     <row r="67" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C67" s="58" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D67" s="68" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="E67" s="62">
         <v>0.42</v>
@@ -7182,10 +7182,10 @@
     </row>
     <row r="68" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C68" s="58" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D68" s="68" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="E68" s="62">
         <v>0.4</v>
@@ -7211,7 +7211,7 @@
     </row>
     <row r="71" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C71" s="193" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="D71" s="114"/>
       <c r="E71" s="114"/>
@@ -7220,7 +7220,7 @@
     </row>
     <row r="72" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C72" s="85" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
     </row>
     <row r="73" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -7228,33 +7228,33 @@
         <v>41</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>43</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
     </row>
     <row r="74" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C74" s="73" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="D74" s="74" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="E74" s="37" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="F74" s="66">
         <v>4</v>
@@ -7273,13 +7273,13 @@
     </row>
     <row r="75" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C75" s="73" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="D75" s="74" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="F75" s="66">
         <v>5</v>
@@ -7298,13 +7298,13 @@
     </row>
     <row r="76" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C76" s="73" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="D76" s="74" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="E76" s="37" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="F76" s="66">
         <v>4</v>
@@ -7323,13 +7323,13 @@
     </row>
     <row r="77" spans="3:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C77" s="73" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="D77" s="74" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="E77" s="37" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="F77" s="66">
         <v>3</v>
@@ -7397,8 +7397,8 @@
       <c r="G2" s="114"/>
     </row>
     <row r="3" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="125" t="s">
-        <v>400</v>
+      <c r="B3" s="133" t="s">
+        <v>394</v>
       </c>
       <c r="C3" s="114"/>
       <c r="D3" s="114"/>
@@ -7443,7 +7443,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="77" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="G6" s="77" t="s">
         <v>12</v>
@@ -7464,10 +7464,10 @@
         <v>15</v>
       </c>
       <c r="E7" s="77" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="F7" s="77" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="G7" s="77" t="s">
         <v>16</v>
@@ -7491,7 +7491,7 @@
         <v>20</v>
       </c>
       <c r="F8" s="77" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="G8" s="77" t="s">
         <v>21</v>
@@ -7515,7 +7515,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="77" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="G9" s="77" t="s">
         <v>26</v>
@@ -7536,10 +7536,10 @@
         <v>29</v>
       </c>
       <c r="E10" s="77" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F10" s="77" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="G10" s="77" t="s">
         <v>30</v>
@@ -7557,7 +7557,7 @@
     </row>
     <row r="12" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="197" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="C12" s="114"/>
       <c r="D12" s="114"/>

</xml_diff>